<commit_message>
feat(hub,inventory): Vendor item code management, UOM matching improvements, invoice workflow updates
- Hub: vendor item code tracking, unmap-code endpoint, improved UOM container matching
- Hub: auto_mapper, auto_send, batch_operations, invoice_status service updates
- Hub: expense items, unmapped items, invoice detail, vendor item detail template updates
- Inventory: units endpoint, item detail, master items, settings, vendor items template updates
- Files: updated Kitchen and Bar Order Sheet

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/files/storage/user_6/Corporate Files/SW Grill Boca Files/General Forms/Kitchen and Bar Order Sheet.xlsx
+++ b/files/storage/user_6/Corporate Files/SW Grill Boca Files/General Forms/Kitchen and Bar Order Sheet.xlsx
@@ -12,7 +12,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">FOOD!$C$1:$I$222</definedName>
     <definedName name="Print_Titles" localSheetId="0">FOOD!$1:$6</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">BAR!$B$1:$I$180</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">BAR!$B$1:$I$178</definedName>
     <definedName name="Print_Titles" localSheetId="1">BAR!$1:$6</definedName>
   </definedNames>
   <calcPr iterateDelta="0.0001"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="381" uniqueCount="381">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="387" uniqueCount="387">
   <si>
     <t xml:space="preserve">SW Grill</t>
   </si>
@@ -697,6 +697,9 @@
     <t>Titos</t>
   </si>
   <si>
+    <t xml:space="preserve">Southern G</t>
+  </si>
+  <si>
     <t>Smirnoff</t>
   </si>
   <si>
@@ -772,9 +775,15 @@
     <t>Empress</t>
   </si>
   <si>
+    <t>RNDC</t>
+  </si>
+  <si>
     <t>Hendricks</t>
   </si>
   <si>
+    <t>Breakthrough</t>
+  </si>
+  <si>
     <t>Whiskey/Scotch</t>
   </si>
   <si>
@@ -934,12 +943,18 @@
     <t xml:space="preserve">Miller Lite</t>
   </si>
   <si>
+    <t xml:space="preserve">Gold Coast</t>
+  </si>
+  <si>
     <t xml:space="preserve">Coors Lite</t>
   </si>
   <si>
     <t xml:space="preserve">Mich Ultra</t>
   </si>
   <si>
+    <t>Bees</t>
+  </si>
+  <si>
     <t xml:space="preserve">Bud Light</t>
   </si>
   <si>
@@ -1060,6 +1075,15 @@
     <t>NAB</t>
   </si>
   <si>
+    <t xml:space="preserve">Bjs or GFS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bjs </t>
+  </si>
+  <si>
+    <t>BJS</t>
+  </si>
+  <si>
     <t xml:space="preserve">Powerade Red</t>
   </si>
   <si>
@@ -1088,12 +1112,6 @@
   </si>
   <si>
     <t xml:space="preserve">Powerade SF Yellow</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bottle Unsweet Tea</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bottle Sweet Tea</t>
   </si>
   <si>
     <t xml:space="preserve">Bottle Coke</t>
@@ -1726,7 +1744,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="145">
+  <cellXfs count="144">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="1" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf fontId="1" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -2079,7 +2097,6 @@
     <xf fontId="9" fillId="2" borderId="20" numFmtId="166" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="24" numFmtId="0" xfId="0" applyBorder="1"/>
     <xf fontId="1" fillId="2" borderId="24" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -7590,11 +7607,13 @@
         <v>2</v>
       </c>
       <c r="H9" s="117"/>
-      <c r="I9" s="120"/>
+      <c r="I9" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="10">
       <c r="B10" s="122" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C10" s="122"/>
       <c r="D10" s="122"/>
@@ -7606,139 +7625,175 @@
         <v>1</v>
       </c>
       <c r="H10" s="123"/>
-      <c r="I10" s="120"/>
+      <c r="I10" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="11">
       <c r="B11" s="122" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C11" s="122"/>
       <c r="D11" s="122"/>
       <c r="E11" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F11" s="118"/>
       <c r="G11" s="119">
         <v>2</v>
       </c>
       <c r="H11" s="123"/>
-      <c r="I11" s="120"/>
+      <c r="I11" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="12">
       <c r="B12" s="122" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C12" s="122"/>
       <c r="D12" s="122"/>
       <c r="E12" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F12" s="118"/>
-      <c r="G12" s="119"/>
+      <c r="G12" s="119">
+        <v>2</v>
+      </c>
       <c r="H12" s="123"/>
-      <c r="I12" s="120"/>
+      <c r="I12" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="13">
       <c r="B13" s="122" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C13" s="122"/>
       <c r="D13" s="122"/>
       <c r="E13" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F13" s="118"/>
-      <c r="G13" s="119"/>
+      <c r="G13" s="119">
+        <v>2</v>
+      </c>
       <c r="H13" s="123"/>
-      <c r="I13" s="120"/>
+      <c r="I13" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="14">
       <c r="B14" s="122" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C14" s="122"/>
       <c r="D14" s="122"/>
       <c r="E14" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F14" s="118"/>
-      <c r="G14" s="119"/>
+      <c r="G14" s="119">
+        <v>2</v>
+      </c>
       <c r="H14" s="123"/>
-      <c r="I14" s="120"/>
+      <c r="I14" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="15">
       <c r="B15" s="122" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C15" s="122"/>
       <c r="D15" s="122"/>
       <c r="E15" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F15" s="118"/>
-      <c r="G15" s="119"/>
+      <c r="G15" s="119">
+        <v>2</v>
+      </c>
       <c r="H15" s="123"/>
-      <c r="I15" s="120"/>
+      <c r="I15" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="16" s="1" customFormat="1">
       <c r="B16" s="122" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C16" s="122"/>
       <c r="D16" s="122"/>
       <c r="E16" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F16" s="118"/>
-      <c r="G16" s="119"/>
+      <c r="G16" s="119">
+        <v>2</v>
+      </c>
       <c r="H16" s="124"/>
-      <c r="I16" s="120"/>
+      <c r="I16" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="17">
       <c r="B17" s="122" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C17" s="122"/>
       <c r="D17" s="122"/>
       <c r="E17" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F17" s="118"/>
-      <c r="G17" s="119"/>
+      <c r="G17" s="119">
+        <v>2</v>
+      </c>
       <c r="H17" s="123"/>
-      <c r="I17" s="120"/>
+      <c r="I17" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="18">
       <c r="B18" s="122" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C18" s="122"/>
       <c r="D18" s="122"/>
       <c r="E18" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F18" s="118"/>
-      <c r="G18" s="119"/>
+      <c r="G18" s="119">
+        <v>2</v>
+      </c>
       <c r="H18" s="123"/>
-      <c r="I18" s="120"/>
+      <c r="I18" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="19">
       <c r="B19" s="122" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C19" s="122"/>
       <c r="D19" s="122"/>
       <c r="E19" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F19" s="118"/>
-      <c r="G19" s="119"/>
+      <c r="G19" s="119">
+        <v>2</v>
+      </c>
       <c r="H19" s="123"/>
-      <c r="I19" s="120"/>
+      <c r="I19" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="20" ht="16.5">
       <c r="B20" s="125" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="C20" s="122"/>
       <c r="D20" s="122"/>
@@ -7750,133 +7805,169 @@
     </row>
     <row r="21">
       <c r="B21" s="122" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C21" s="122"/>
       <c r="D21" s="122"/>
       <c r="E21" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F21" s="118"/>
-      <c r="G21" s="119"/>
+      <c r="G21" s="119">
+        <v>2</v>
+      </c>
       <c r="H21" s="117"/>
-      <c r="I21" s="120"/>
+      <c r="I21" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="22">
       <c r="B22" s="122" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C22" s="122"/>
       <c r="D22" s="122"/>
       <c r="E22" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F22" s="118"/>
-      <c r="G22" s="119"/>
+      <c r="G22" s="119">
+        <v>3</v>
+      </c>
       <c r="H22" s="123"/>
-      <c r="I22" s="120"/>
+      <c r="I22" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="23">
       <c r="B23" s="122" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C23" s="122"/>
       <c r="D23" s="122"/>
       <c r="E23" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F23" s="118"/>
-      <c r="G23" s="119"/>
+      <c r="G23" s="119">
+        <v>2</v>
+      </c>
       <c r="H23" s="123"/>
-      <c r="I23" s="120"/>
+      <c r="I23" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="24">
       <c r="B24" s="126" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C24" s="126"/>
       <c r="D24" s="126"/>
       <c r="E24" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F24" s="118"/>
-      <c r="G24" s="119"/>
+      <c r="G24" s="119">
+        <v>2</v>
+      </c>
       <c r="H24" s="123"/>
-      <c r="I24" s="120"/>
+      <c r="I24" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="25">
       <c r="B25" s="126" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C25" s="126"/>
       <c r="D25" s="126"/>
       <c r="E25" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F25" s="118"/>
-      <c r="G25" s="119"/>
+      <c r="G25" s="119">
+        <v>3</v>
+      </c>
       <c r="H25" s="123"/>
-      <c r="I25" s="120"/>
+      <c r="I25" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="26">
       <c r="B26" s="126" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="C26" s="126"/>
       <c r="D26" s="126"/>
       <c r="E26" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F26" s="118"/>
-      <c r="G26" s="119"/>
+      <c r="G26" s="119">
+        <v>2</v>
+      </c>
       <c r="H26" s="123"/>
-      <c r="I26" s="120"/>
+      <c r="I26" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="27">
       <c r="B27" s="126" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C27" s="126"/>
       <c r="D27" s="126"/>
       <c r="E27" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F27" s="118"/>
-      <c r="G27" s="119"/>
+      <c r="G27" s="119">
+        <v>2</v>
+      </c>
       <c r="H27" s="123"/>
-      <c r="I27" s="120"/>
+      <c r="I27" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="28">
       <c r="B28" s="126" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C28" s="126"/>
       <c r="D28" s="126"/>
       <c r="E28" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F28" s="118"/>
-      <c r="G28" s="119"/>
+      <c r="G28" s="119">
+        <v>2</v>
+      </c>
       <c r="H28" s="123"/>
-      <c r="I28" s="120"/>
+      <c r="I28" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="29">
       <c r="B29" s="126" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C29" s="126"/>
       <c r="D29" s="126"/>
       <c r="E29" s="117" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="F29" s="118"/>
-      <c r="G29" s="119"/>
+      <c r="G29" s="119">
+        <v>1</v>
+      </c>
       <c r="H29" s="123"/>
-      <c r="I29" s="120"/>
+      <c r="I29" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="30" ht="16.5">
       <c r="B30" s="127" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C30" s="126"/>
       <c r="D30" s="126"/>
@@ -7888,63 +7979,79 @@
     </row>
     <row r="31">
       <c r="B31" s="126" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C31" s="126"/>
       <c r="D31" s="126"/>
       <c r="E31" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F31" s="118"/>
-      <c r="G31" s="119"/>
+      <c r="G31" s="119">
+        <v>2</v>
+      </c>
       <c r="H31" s="123"/>
-      <c r="I31" s="120"/>
+      <c r="I31" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="32">
       <c r="B32" s="126" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C32" s="126"/>
       <c r="D32" s="126"/>
       <c r="E32" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F32" s="118"/>
-      <c r="G32" s="119"/>
+      <c r="G32" s="119">
+        <v>3</v>
+      </c>
       <c r="H32" s="123"/>
-      <c r="I32" s="120"/>
+      <c r="I32" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="33">
       <c r="B33" s="128" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C33" s="128"/>
       <c r="D33" s="128"/>
       <c r="E33" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F33" s="118"/>
-      <c r="G33" s="119"/>
+      <c r="G33" s="119">
+        <v>2</v>
+      </c>
       <c r="H33" s="123"/>
-      <c r="I33" s="120"/>
+      <c r="I33" s="120" t="s">
+        <v>250</v>
+      </c>
     </row>
     <row r="34">
       <c r="B34" s="128" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="C34" s="128"/>
       <c r="D34" s="128"/>
       <c r="E34" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F34" s="118"/>
-      <c r="G34" s="119"/>
+      <c r="G34" s="119">
+        <v>2</v>
+      </c>
       <c r="H34" s="123"/>
-      <c r="I34" s="120"/>
+      <c r="I34" s="120" t="s">
+        <v>252</v>
+      </c>
     </row>
     <row r="35" ht="16.5">
       <c r="B35" s="129" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="C35" s="128"/>
       <c r="D35" s="128"/>
@@ -7956,7 +8063,7 @@
     </row>
     <row r="36">
       <c r="B36" s="128" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="C36" s="128"/>
       <c r="D36" s="128"/>
@@ -7964,279 +8071,357 @@
         <v>222</v>
       </c>
       <c r="F36" s="118"/>
-      <c r="G36" s="119"/>
+      <c r="G36" s="119">
+        <v>1</v>
+      </c>
       <c r="H36" s="123"/>
-      <c r="I36" s="120"/>
+      <c r="I36" s="120" t="s">
+        <v>252</v>
+      </c>
     </row>
     <row r="37">
       <c r="B37" s="128" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="C37" s="128"/>
       <c r="D37" s="128"/>
       <c r="E37" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F37" s="118"/>
-      <c r="G37" s="119"/>
+      <c r="G37" s="119">
+        <v>2</v>
+      </c>
       <c r="H37" s="123"/>
-      <c r="I37" s="120"/>
+      <c r="I37" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="38">
       <c r="B38" s="128" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="C38" s="128"/>
       <c r="D38" s="128"/>
       <c r="E38" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F38" s="118"/>
-      <c r="G38" s="119"/>
+      <c r="G38" s="119">
+        <v>2</v>
+      </c>
       <c r="H38" s="123"/>
-      <c r="I38" s="120"/>
+      <c r="I38" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="39">
       <c r="B39" s="128" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="C39" s="128"/>
       <c r="D39" s="128"/>
       <c r="E39" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F39" s="118"/>
-      <c r="G39" s="119"/>
+      <c r="G39" s="119">
+        <v>2</v>
+      </c>
       <c r="H39" s="123"/>
-      <c r="I39" s="120"/>
+      <c r="I39" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="40">
       <c r="B40" s="128" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="C40" s="128"/>
       <c r="D40" s="128"/>
       <c r="E40" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F40" s="118"/>
-      <c r="G40" s="119"/>
+      <c r="G40" s="119">
+        <v>2</v>
+      </c>
       <c r="H40" s="123"/>
-      <c r="I40" s="120"/>
+      <c r="I40" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="41">
       <c r="B41" s="128" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="C41" s="128"/>
       <c r="D41" s="128"/>
       <c r="E41" s="117" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="F41" s="118"/>
-      <c r="G41" s="119"/>
+      <c r="G41" s="119">
+        <v>1</v>
+      </c>
       <c r="H41" s="123"/>
-      <c r="I41" s="120"/>
+      <c r="I41" s="120" t="s">
+        <v>252</v>
+      </c>
     </row>
     <row r="42">
       <c r="B42" s="128" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="C42" s="128"/>
       <c r="D42" s="128"/>
       <c r="E42" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F42" s="118"/>
-      <c r="G42" s="119"/>
+      <c r="G42" s="119">
+        <v>4</v>
+      </c>
       <c r="H42" s="123"/>
-      <c r="I42" s="120"/>
+      <c r="I42" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="43">
       <c r="B43" s="128" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="C43" s="128"/>
       <c r="D43" s="128"/>
       <c r="E43" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F43" s="118"/>
-      <c r="G43" s="119"/>
+      <c r="G43" s="119">
+        <v>2</v>
+      </c>
       <c r="H43" s="123"/>
-      <c r="I43" s="120"/>
+      <c r="I43" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="44">
       <c r="B44" s="128" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="C44" s="128"/>
       <c r="D44" s="128"/>
       <c r="E44" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F44" s="118"/>
-      <c r="G44" s="119"/>
+      <c r="G44" s="119">
+        <v>2</v>
+      </c>
       <c r="H44" s="123"/>
-      <c r="I44" s="120"/>
+      <c r="I44" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="45">
       <c r="B45" s="128" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="C45" s="128"/>
       <c r="D45" s="128"/>
       <c r="E45" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F45" s="118"/>
-      <c r="G45" s="119"/>
+      <c r="G45" s="119">
+        <v>2</v>
+      </c>
       <c r="H45" s="123"/>
-      <c r="I45" s="120"/>
+      <c r="I45" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="46">
       <c r="B46" s="128" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="C46" s="128"/>
       <c r="D46" s="128"/>
       <c r="E46" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F46" s="118"/>
-      <c r="G46" s="119"/>
+      <c r="G46" s="119">
+        <v>2</v>
+      </c>
       <c r="H46" s="123"/>
-      <c r="I46" s="120"/>
+      <c r="I46" s="120" t="s">
+        <v>252</v>
+      </c>
     </row>
     <row r="47">
       <c r="B47" s="128" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="C47" s="128"/>
       <c r="D47" s="128"/>
       <c r="E47" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F47" s="118"/>
-      <c r="G47" s="119"/>
+      <c r="G47" s="119">
+        <v>2</v>
+      </c>
       <c r="H47" s="123"/>
-      <c r="I47" s="120"/>
+      <c r="I47" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="48">
       <c r="B48" s="128" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="C48" s="128"/>
       <c r="D48" s="128"/>
       <c r="E48" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F48" s="118"/>
-      <c r="G48" s="119"/>
+      <c r="G48" s="119">
+        <v>2</v>
+      </c>
       <c r="H48" s="123"/>
-      <c r="I48" s="120"/>
+      <c r="I48" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="49">
       <c r="B49" s="128" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="C49" s="128"/>
       <c r="D49" s="128"/>
       <c r="E49" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F49" s="118"/>
-      <c r="G49" s="119"/>
+      <c r="G49" s="119">
+        <v>1</v>
+      </c>
       <c r="H49" s="123"/>
       <c r="I49" s="120"/>
     </row>
     <row r="50">
       <c r="B50" s="128" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="C50" s="128"/>
       <c r="D50" s="128"/>
       <c r="E50" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F50" s="118"/>
-      <c r="G50" s="119"/>
+      <c r="G50" s="119">
+        <v>1</v>
+      </c>
       <c r="H50" s="123"/>
-      <c r="I50" s="120"/>
+      <c r="I50" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="51">
       <c r="B51" s="128" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="C51" s="128"/>
       <c r="D51" s="128"/>
       <c r="E51" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F51" s="118"/>
-      <c r="G51" s="119"/>
+      <c r="G51" s="119">
+        <v>1</v>
+      </c>
       <c r="H51" s="123"/>
-      <c r="I51" s="120"/>
+      <c r="I51" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="52">
       <c r="B52" s="128" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="C52" s="128"/>
       <c r="D52" s="128"/>
       <c r="E52" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F52" s="118"/>
-      <c r="G52" s="119"/>
+      <c r="G52" s="119">
+        <v>2</v>
+      </c>
       <c r="H52" s="123"/>
-      <c r="I52" s="120"/>
+      <c r="I52" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="53">
       <c r="B53" s="128" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="C53" s="128"/>
       <c r="D53" s="128"/>
       <c r="E53" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F53" s="118"/>
-      <c r="G53" s="119"/>
+      <c r="G53" s="119">
+        <v>1</v>
+      </c>
       <c r="H53" s="123"/>
-      <c r="I53" s="120"/>
+      <c r="I53" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="54">
       <c r="B54" s="128" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="C54" s="128"/>
       <c r="D54" s="128"/>
       <c r="E54" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F54" s="118"/>
-      <c r="G54" s="119"/>
+      <c r="G54" s="119">
+        <v>2</v>
+      </c>
       <c r="H54" s="123"/>
-      <c r="I54" s="120"/>
+      <c r="I54" s="120" t="s">
+        <v>250</v>
+      </c>
     </row>
     <row r="55">
       <c r="B55" s="128" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="C55" s="128"/>
       <c r="D55" s="128"/>
       <c r="E55" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F55" s="118"/>
-      <c r="G55" s="119"/>
+      <c r="G55" s="119">
+        <v>1</v>
+      </c>
       <c r="H55" s="123"/>
-      <c r="I55" s="120"/>
+      <c r="I55" s="120" t="s">
+        <v>250</v>
+      </c>
     </row>
     <row r="56" ht="16.5">
       <c r="B56" s="129" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="C56" s="129"/>
       <c r="D56" s="128"/>
@@ -8248,77 +8433,97 @@
     </row>
     <row r="57">
       <c r="B57" s="128" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="C57" s="128"/>
       <c r="D57" s="128"/>
       <c r="E57" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F57" s="118"/>
-      <c r="G57" s="119"/>
+      <c r="G57" s="119">
+        <v>2</v>
+      </c>
       <c r="H57" s="123"/>
-      <c r="I57" s="120"/>
+      <c r="I57" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="58">
       <c r="B58" s="128" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="C58" s="128"/>
       <c r="D58" s="128"/>
       <c r="E58" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F58" s="118"/>
-      <c r="G58" s="119"/>
+      <c r="G58" s="119">
+        <v>4</v>
+      </c>
       <c r="H58" s="123"/>
-      <c r="I58" s="120"/>
+      <c r="I58" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="59">
       <c r="B59" s="128" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="C59" s="128"/>
       <c r="D59" s="128"/>
       <c r="E59" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F59" s="118"/>
-      <c r="G59" s="119"/>
+      <c r="G59" s="119">
+        <v>1</v>
+      </c>
       <c r="H59" s="123"/>
-      <c r="I59" s="120"/>
+      <c r="I59" s="120" t="s">
+        <v>250</v>
+      </c>
     </row>
     <row r="60">
       <c r="B60" s="128" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="C60" s="128"/>
       <c r="D60" s="128"/>
       <c r="E60" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F60" s="118"/>
-      <c r="G60" s="119"/>
+      <c r="G60" s="119">
+        <v>1</v>
+      </c>
       <c r="H60" s="123"/>
-      <c r="I60" s="120"/>
+      <c r="I60" s="120" t="s">
+        <v>250</v>
+      </c>
     </row>
     <row r="61">
       <c r="B61" s="128" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="C61" s="128"/>
       <c r="D61" s="128"/>
       <c r="E61" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F61" s="118"/>
-      <c r="G61" s="119"/>
+      <c r="G61" s="119">
+        <v>1</v>
+      </c>
       <c r="H61" s="123"/>
-      <c r="I61" s="120"/>
+      <c r="I61" s="120" t="s">
+        <v>250</v>
+      </c>
     </row>
     <row r="62" ht="16.5">
       <c r="B62" s="129" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="C62" s="128"/>
       <c r="D62" s="128"/>
@@ -8330,119 +8535,151 @@
     </row>
     <row r="63">
       <c r="B63" s="128" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="C63" s="128"/>
       <c r="D63" s="128"/>
       <c r="E63" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F63" s="118"/>
-      <c r="G63" s="119"/>
+      <c r="G63" s="119">
+        <v>1</v>
+      </c>
       <c r="H63" s="123"/>
-      <c r="I63" s="120"/>
+      <c r="I63" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="64">
       <c r="B64" s="128" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="C64" s="128"/>
       <c r="D64" s="128"/>
       <c r="E64" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F64" s="118"/>
-      <c r="G64" s="119"/>
+      <c r="G64" s="119">
+        <v>2</v>
+      </c>
       <c r="H64" s="123"/>
-      <c r="I64" s="120"/>
+      <c r="I64" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="65">
       <c r="B65" s="128" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="C65" s="128"/>
       <c r="D65" s="128"/>
       <c r="E65" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F65" s="118"/>
-      <c r="G65" s="119"/>
+      <c r="G65" s="119">
+        <v>2</v>
+      </c>
       <c r="H65" s="123"/>
-      <c r="I65" s="120"/>
+      <c r="I65" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="66">
       <c r="B66" s="128" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="C66" s="128"/>
       <c r="D66" s="128"/>
       <c r="E66" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F66" s="118"/>
-      <c r="G66" s="119"/>
+      <c r="G66" s="119">
+        <v>1</v>
+      </c>
       <c r="H66" s="123"/>
-      <c r="I66" s="120"/>
+      <c r="I66" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="67">
       <c r="B67" s="128" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="C67" s="128"/>
       <c r="D67" s="128"/>
       <c r="E67" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F67" s="118"/>
-      <c r="G67" s="119"/>
+      <c r="G67" s="119">
+        <v>1</v>
+      </c>
       <c r="H67" s="123"/>
-      <c r="I67" s="120"/>
+      <c r="I67" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="68">
       <c r="B68" s="128" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="C68" s="128"/>
       <c r="D68" s="128"/>
       <c r="E68" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F68" s="118"/>
-      <c r="G68" s="119"/>
+      <c r="G68" s="119">
+        <v>3</v>
+      </c>
       <c r="H68" s="123"/>
-      <c r="I68" s="120"/>
+      <c r="I68" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="69">
       <c r="B69" s="128" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="C69" s="128"/>
       <c r="D69" s="128"/>
       <c r="E69" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F69" s="118"/>
-      <c r="G69" s="119"/>
+      <c r="G69" s="119">
+        <v>3</v>
+      </c>
       <c r="H69" s="123"/>
-      <c r="I69" s="120"/>
+      <c r="I69" s="120" t="s">
+        <v>252</v>
+      </c>
     </row>
     <row r="70">
       <c r="B70" s="128" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="C70" s="128"/>
       <c r="D70" s="128"/>
       <c r="E70" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F70" s="118"/>
-      <c r="G70" s="119"/>
+      <c r="G70" s="119">
+        <v>1</v>
+      </c>
       <c r="H70" s="123"/>
-      <c r="I70" s="120"/>
+      <c r="I70" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="71">
       <c r="B71" s="128" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="C71" s="128"/>
       <c r="D71" s="128"/>
@@ -8450,13 +8687,17 @@
         <v>222</v>
       </c>
       <c r="F71" s="118"/>
-      <c r="G71" s="119"/>
+      <c r="G71" s="119">
+        <v>1</v>
+      </c>
       <c r="H71" s="123"/>
-      <c r="I71" s="120"/>
+      <c r="I71" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="72">
       <c r="B72" s="128" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="C72" s="128"/>
       <c r="D72" s="128"/>
@@ -8464,13 +8705,17 @@
         <v>222</v>
       </c>
       <c r="F72" s="118"/>
-      <c r="G72" s="119"/>
+      <c r="G72" s="119">
+        <v>1</v>
+      </c>
       <c r="H72" s="123"/>
-      <c r="I72" s="120"/>
+      <c r="I72" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="73">
       <c r="B73" s="128" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="C73" s="128"/>
       <c r="D73" s="128"/>
@@ -8478,111 +8723,143 @@
         <v>222</v>
       </c>
       <c r="F73" s="118"/>
-      <c r="G73" s="119"/>
+      <c r="G73" s="119">
+        <v>1</v>
+      </c>
       <c r="H73" s="123"/>
-      <c r="I73" s="120"/>
+      <c r="I73" s="120" t="s">
+        <v>250</v>
+      </c>
     </row>
     <row r="74">
       <c r="B74" s="128" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="C74" s="128"/>
       <c r="D74" s="128"/>
       <c r="E74" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F74" s="118"/>
-      <c r="G74" s="119"/>
+      <c r="G74" s="119">
+        <v>1</v>
+      </c>
       <c r="H74" s="123"/>
-      <c r="I74" s="120"/>
+      <c r="I74" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="75">
       <c r="B75" s="128" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="C75" s="128"/>
       <c r="D75" s="128"/>
       <c r="E75" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F75" s="118"/>
-      <c r="G75" s="119"/>
+      <c r="G75" s="119">
+        <v>1</v>
+      </c>
       <c r="H75" s="123"/>
-      <c r="I75" s="120"/>
+      <c r="I75" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="76">
       <c r="B76" s="128" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="C76" s="128"/>
       <c r="D76" s="128"/>
       <c r="E76" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F76" s="118"/>
-      <c r="G76" s="119"/>
+      <c r="G76" s="119">
+        <v>1</v>
+      </c>
       <c r="H76" s="123"/>
-      <c r="I76" s="120"/>
+      <c r="I76" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="77">
       <c r="B77" s="128" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="C77" s="128"/>
       <c r="D77" s="128"/>
       <c r="E77" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F77" s="118"/>
-      <c r="G77" s="119"/>
+      <c r="G77" s="119">
+        <v>1</v>
+      </c>
       <c r="H77" s="123"/>
-      <c r="I77" s="120"/>
+      <c r="I77" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="78">
       <c r="B78" s="128" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="C78" s="128"/>
       <c r="D78" s="128"/>
       <c r="E78" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F78" s="118"/>
-      <c r="G78" s="119"/>
+      <c r="G78" s="119">
+        <v>1</v>
+      </c>
       <c r="H78" s="123"/>
-      <c r="I78" s="120"/>
+      <c r="I78" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="79">
       <c r="B79" s="128" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="C79" s="128"/>
       <c r="D79" s="128"/>
       <c r="E79" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F79" s="118"/>
-      <c r="G79" s="119"/>
+      <c r="G79" s="119">
+        <v>1</v>
+      </c>
       <c r="H79" s="123"/>
-      <c r="I79" s="120"/>
+      <c r="I79" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="80">
       <c r="B80" s="128" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="C80" s="128"/>
       <c r="D80" s="128"/>
       <c r="E80" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F80" s="118"/>
-      <c r="G80" s="119"/>
+      <c r="G80" s="119">
+        <v>2</v>
+      </c>
       <c r="H80" s="123"/>
-      <c r="I80" s="120"/>
+      <c r="I80" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="81">
       <c r="B81" s="128" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="C81" s="128"/>
       <c r="D81" s="128"/>
@@ -8590,55 +8867,71 @@
         <v>222</v>
       </c>
       <c r="F81" s="118"/>
-      <c r="G81" s="119"/>
+      <c r="G81" s="119">
+        <v>1</v>
+      </c>
       <c r="H81" s="123"/>
-      <c r="I81" s="120"/>
+      <c r="I81" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="82">
       <c r="B82" s="128" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="C82" s="128"/>
       <c r="D82" s="128"/>
       <c r="E82" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F82" s="118"/>
-      <c r="G82" s="119"/>
+      <c r="G82" s="119">
+        <v>1</v>
+      </c>
       <c r="H82" s="123"/>
-      <c r="I82" s="120"/>
+      <c r="I82" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="83">
       <c r="B83" s="128" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="C83" s="128"/>
       <c r="D83" s="128"/>
       <c r="E83" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F83" s="118"/>
-      <c r="G83" s="119"/>
+      <c r="G83" s="119">
+        <v>1</v>
+      </c>
       <c r="H83" s="123"/>
-      <c r="I83" s="120"/>
+      <c r="I83" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="84">
       <c r="B84" s="128" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="C84" s="128"/>
       <c r="D84" s="128"/>
       <c r="E84" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F84" s="118"/>
-      <c r="G84" s="119"/>
+      <c r="G84" s="119">
+        <v>1</v>
+      </c>
       <c r="H84" s="123"/>
-      <c r="I84" s="120"/>
+      <c r="I84" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="85">
       <c r="B85" s="130" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="C85" s="130"/>
       <c r="D85" s="130"/>
@@ -8646,13 +8939,17 @@
         <v>222</v>
       </c>
       <c r="F85" s="118"/>
-      <c r="G85" s="119"/>
+      <c r="G85" s="119">
+        <v>1</v>
+      </c>
       <c r="H85" s="123"/>
-      <c r="I85" s="120"/>
+      <c r="I85" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="86" ht="15" customHeight="1">
       <c r="B86" s="44" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="C86" s="44"/>
       <c r="D86" s="44"/>
@@ -8682,7 +8979,7 @@
     </row>
     <row r="88">
       <c r="B88" s="132" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="C88" s="132"/>
       <c r="D88" s="132"/>
@@ -8690,13 +8987,17 @@
         <v>222</v>
       </c>
       <c r="F88" s="118"/>
-      <c r="G88" s="133"/>
+      <c r="G88" s="133">
+        <v>10</v>
+      </c>
       <c r="H88" s="123"/>
-      <c r="I88" s="120"/>
+      <c r="I88" s="120" t="s">
+        <v>306</v>
+      </c>
     </row>
     <row r="89">
       <c r="B89" s="126" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="C89" s="126"/>
       <c r="D89" s="126"/>
@@ -8704,13 +9005,17 @@
         <v>222</v>
       </c>
       <c r="F89" s="118"/>
-      <c r="G89" s="133"/>
+      <c r="G89" s="133">
+        <v>10</v>
+      </c>
       <c r="H89" s="123"/>
-      <c r="I89" s="120"/>
+      <c r="I89" s="120" t="s">
+        <v>306</v>
+      </c>
     </row>
     <row r="90">
       <c r="B90" s="126" t="s">
-        <v>304</v>
+        <v>308</v>
       </c>
       <c r="C90" s="126"/>
       <c r="D90" s="126"/>
@@ -8718,13 +9023,17 @@
         <v>222</v>
       </c>
       <c r="F90" s="118"/>
-      <c r="G90" s="133"/>
+      <c r="G90" s="133">
+        <v>6</v>
+      </c>
       <c r="H90" s="123"/>
-      <c r="I90" s="120"/>
+      <c r="I90" s="120" t="s">
+        <v>309</v>
+      </c>
     </row>
     <row r="91">
       <c r="B91" s="122" t="s">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="C91" s="122"/>
       <c r="D91" s="122"/>
@@ -8732,13 +9041,17 @@
         <v>222</v>
       </c>
       <c r="F91" s="118"/>
-      <c r="G91" s="133"/>
+      <c r="G91" s="133">
+        <v>3</v>
+      </c>
       <c r="H91" s="123"/>
-      <c r="I91" s="120"/>
+      <c r="I91" s="120" t="s">
+        <v>309</v>
+      </c>
     </row>
     <row r="92">
       <c r="B92" s="122" t="s">
-        <v>306</v>
+        <v>311</v>
       </c>
       <c r="C92" s="122"/>
       <c r="D92" s="122"/>
@@ -8746,13 +9059,17 @@
         <v>222</v>
       </c>
       <c r="F92" s="118"/>
-      <c r="G92" s="133"/>
+      <c r="G92" s="133">
+        <v>2</v>
+      </c>
       <c r="H92" s="123"/>
-      <c r="I92" s="120"/>
+      <c r="I92" s="120" t="s">
+        <v>309</v>
+      </c>
     </row>
     <row r="93">
       <c r="B93" s="122" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="C93" s="122"/>
       <c r="D93" s="122"/>
@@ -8760,13 +9077,17 @@
         <v>222</v>
       </c>
       <c r="F93" s="118"/>
-      <c r="G93" s="133"/>
+      <c r="G93" s="133">
+        <v>6</v>
+      </c>
       <c r="H93" s="123"/>
-      <c r="I93" s="120"/>
+      <c r="I93" s="120" t="s">
+        <v>309</v>
+      </c>
     </row>
     <row r="94">
       <c r="B94" s="122" t="s">
-        <v>308</v>
+        <v>313</v>
       </c>
       <c r="C94" s="122"/>
       <c r="D94" s="122"/>
@@ -8774,13 +9095,17 @@
         <v>222</v>
       </c>
       <c r="F94" s="118"/>
-      <c r="G94" s="133"/>
+      <c r="G94" s="133">
+        <v>6</v>
+      </c>
       <c r="H94" s="123"/>
-      <c r="I94" s="120"/>
+      <c r="I94" s="120" t="s">
+        <v>309</v>
+      </c>
     </row>
     <row r="95">
       <c r="B95" s="122" t="s">
-        <v>309</v>
+        <v>314</v>
       </c>
       <c r="C95" s="122"/>
       <c r="D95" s="122"/>
@@ -8788,13 +9113,17 @@
         <v>222</v>
       </c>
       <c r="F95" s="118"/>
-      <c r="G95" s="133"/>
+      <c r="G95" s="133">
+        <v>4</v>
+      </c>
       <c r="H95" s="123"/>
-      <c r="I95" s="120"/>
+      <c r="I95" s="120" t="s">
+        <v>306</v>
+      </c>
     </row>
     <row r="96">
-      <c r="B96" s="134" t="s">
-        <v>310</v>
+      <c r="B96" s="122" t="s">
+        <v>315</v>
       </c>
       <c r="C96" s="122"/>
       <c r="D96" s="122"/>
@@ -8802,13 +9131,17 @@
         <v>222</v>
       </c>
       <c r="F96" s="118"/>
-      <c r="G96" s="133"/>
+      <c r="G96" s="133">
+        <v>2</v>
+      </c>
       <c r="H96" s="123"/>
-      <c r="I96" s="120"/>
+      <c r="I96" s="120" t="s">
+        <v>306</v>
+      </c>
     </row>
     <row r="97">
       <c r="B97" s="122" t="s">
-        <v>311</v>
+        <v>316</v>
       </c>
       <c r="C97" s="122"/>
       <c r="D97" s="122"/>
@@ -8816,13 +9149,17 @@
         <v>222</v>
       </c>
       <c r="F97" s="118"/>
-      <c r="G97" s="133"/>
+      <c r="G97" s="133">
+        <v>6</v>
+      </c>
       <c r="H97" s="123"/>
-      <c r="I97" s="120"/>
+      <c r="I97" s="120" t="s">
+        <v>309</v>
+      </c>
     </row>
     <row r="98">
       <c r="B98" s="122" t="s">
-        <v>312</v>
+        <v>317</v>
       </c>
       <c r="C98" s="122"/>
       <c r="D98" s="122"/>
@@ -8830,13 +9167,17 @@
         <v>222</v>
       </c>
       <c r="F98" s="118"/>
-      <c r="G98" s="133"/>
+      <c r="G98" s="133">
+        <v>8</v>
+      </c>
       <c r="H98" s="123"/>
-      <c r="I98" s="120"/>
+      <c r="I98" s="120" t="s">
+        <v>306</v>
+      </c>
     </row>
     <row r="99">
       <c r="B99" s="122" t="s">
-        <v>313</v>
+        <v>318</v>
       </c>
       <c r="C99" s="122"/>
       <c r="D99" s="122"/>
@@ -8844,13 +9185,17 @@
         <v>222</v>
       </c>
       <c r="F99" s="118"/>
-      <c r="G99" s="133"/>
+      <c r="G99" s="133">
+        <v>8</v>
+      </c>
       <c r="H99" s="123"/>
-      <c r="I99" s="120"/>
+      <c r="I99" s="120" t="s">
+        <v>306</v>
+      </c>
     </row>
     <row r="100">
       <c r="B100" s="126" t="s">
-        <v>314</v>
+        <v>319</v>
       </c>
       <c r="C100" s="126"/>
       <c r="D100" s="126"/>
@@ -8858,13 +9203,17 @@
         <v>222</v>
       </c>
       <c r="F100" s="118"/>
-      <c r="G100" s="133"/>
+      <c r="G100" s="133">
+        <v>2</v>
+      </c>
       <c r="H100" s="123"/>
-      <c r="I100" s="120"/>
+      <c r="I100" s="120" t="s">
+        <v>306</v>
+      </c>
     </row>
     <row r="101" ht="15" customHeight="1">
       <c r="B101" s="44" t="s">
-        <v>315</v>
+        <v>320</v>
       </c>
       <c r="C101" s="44"/>
       <c r="D101" s="44"/>
@@ -8894,7 +9243,7 @@
     </row>
     <row r="103">
       <c r="B103" s="132" t="s">
-        <v>316</v>
+        <v>321</v>
       </c>
       <c r="C103" s="132"/>
       <c r="D103" s="132"/>
@@ -8902,13 +9251,17 @@
         <v>222</v>
       </c>
       <c r="F103" s="118"/>
-      <c r="G103" s="133"/>
+      <c r="G103" s="133">
+        <v>2</v>
+      </c>
       <c r="H103" s="123"/>
-      <c r="I103" s="120"/>
+      <c r="I103" s="120" t="s">
+        <v>252</v>
+      </c>
     </row>
     <row r="104">
       <c r="B104" s="126" t="s">
-        <v>317</v>
+        <v>322</v>
       </c>
       <c r="C104" s="126"/>
       <c r="D104" s="126"/>
@@ -8916,125 +9269,161 @@
         <v>222</v>
       </c>
       <c r="F104" s="118"/>
-      <c r="G104" s="133"/>
+      <c r="G104" s="133">
+        <v>2</v>
+      </c>
       <c r="H104" s="123"/>
-      <c r="I104" s="120"/>
+      <c r="I104" s="120" t="s">
+        <v>252</v>
+      </c>
     </row>
     <row r="105">
       <c r="B105" s="126" t="s">
-        <v>318</v>
-      </c>
-      <c r="C105" s="135"/>
-      <c r="D105" s="135"/>
+        <v>323</v>
+      </c>
+      <c r="C105" s="134"/>
+      <c r="D105" s="134"/>
       <c r="E105" s="117" t="s">
         <v>222</v>
       </c>
       <c r="F105" s="118"/>
-      <c r="G105" s="133"/>
+      <c r="G105" s="133">
+        <v>2</v>
+      </c>
       <c r="H105" s="123"/>
-      <c r="I105" s="120"/>
+      <c r="I105" s="120" t="s">
+        <v>252</v>
+      </c>
     </row>
     <row r="106">
       <c r="B106" s="126" t="s">
-        <v>319</v>
-      </c>
-      <c r="C106" s="135"/>
-      <c r="D106" s="135"/>
+        <v>324</v>
+      </c>
+      <c r="C106" s="134"/>
+      <c r="D106" s="134"/>
       <c r="E106" s="117" t="s">
         <v>222</v>
       </c>
       <c r="F106" s="118"/>
-      <c r="G106" s="133"/>
+      <c r="G106" s="133">
+        <v>2</v>
+      </c>
       <c r="H106" s="123"/>
-      <c r="I106" s="120"/>
+      <c r="I106" s="120" t="s">
+        <v>252</v>
+      </c>
     </row>
     <row r="107">
       <c r="B107" s="126" t="s">
-        <v>320</v>
-      </c>
-      <c r="C107" s="135"/>
-      <c r="D107" s="135"/>
+        <v>325</v>
+      </c>
+      <c r="C107" s="134"/>
+      <c r="D107" s="134"/>
       <c r="E107" s="117" t="s">
         <v>222</v>
       </c>
       <c r="F107" s="118"/>
-      <c r="G107" s="133"/>
+      <c r="G107" s="133">
+        <v>2</v>
+      </c>
       <c r="H107" s="123"/>
-      <c r="I107" s="120"/>
+      <c r="I107" s="120" t="s">
+        <v>252</v>
+      </c>
     </row>
     <row r="108">
       <c r="B108" s="126" t="s">
-        <v>321</v>
-      </c>
-      <c r="C108" s="135"/>
-      <c r="D108" s="135"/>
+        <v>326</v>
+      </c>
+      <c r="C108" s="134"/>
+      <c r="D108" s="134"/>
       <c r="E108" s="117" t="s">
         <v>222</v>
       </c>
       <c r="F108" s="118"/>
-      <c r="G108" s="133"/>
+      <c r="G108" s="133">
+        <v>2</v>
+      </c>
       <c r="H108" s="123"/>
-      <c r="I108" s="120"/>
+      <c r="I108" s="120" t="s">
+        <v>252</v>
+      </c>
     </row>
     <row r="109">
       <c r="B109" s="126" t="s">
-        <v>322</v>
-      </c>
-      <c r="C109" s="135"/>
-      <c r="D109" s="135"/>
+        <v>327</v>
+      </c>
+      <c r="C109" s="134"/>
+      <c r="D109" s="134"/>
       <c r="E109" s="117" t="s">
         <v>222</v>
       </c>
       <c r="F109" s="118"/>
-      <c r="G109" s="133"/>
+      <c r="G109" s="133">
+        <v>2</v>
+      </c>
       <c r="H109" s="123"/>
-      <c r="I109" s="120"/>
+      <c r="I109" s="120" t="s">
+        <v>252</v>
+      </c>
     </row>
     <row r="110">
       <c r="B110" s="126" t="s">
-        <v>323</v>
-      </c>
-      <c r="C110" s="135"/>
-      <c r="D110" s="135"/>
+        <v>328</v>
+      </c>
+      <c r="C110" s="134"/>
+      <c r="D110" s="134"/>
       <c r="E110" s="117" t="s">
         <v>222</v>
       </c>
       <c r="F110" s="118"/>
-      <c r="G110" s="133"/>
+      <c r="G110" s="133">
+        <v>3</v>
+      </c>
       <c r="H110" s="123"/>
-      <c r="I110" s="120"/>
+      <c r="I110" s="120" t="s">
+        <v>306</v>
+      </c>
     </row>
     <row r="111">
       <c r="B111" s="126" t="s">
-        <v>324</v>
-      </c>
-      <c r="C111" s="135"/>
-      <c r="D111" s="135"/>
+        <v>329</v>
+      </c>
+      <c r="C111" s="134"/>
+      <c r="D111" s="134"/>
       <c r="E111" s="117" t="s">
         <v>222</v>
       </c>
       <c r="F111" s="118"/>
-      <c r="G111" s="133"/>
+      <c r="G111" s="133">
+        <v>3</v>
+      </c>
       <c r="H111" s="123"/>
-      <c r="I111" s="120"/>
+      <c r="I111" s="120" t="s">
+        <v>306</v>
+      </c>
     </row>
     <row r="112">
       <c r="B112" s="126" t="s">
-        <v>325</v>
-      </c>
-      <c r="C112" s="135"/>
-      <c r="D112" s="135"/>
+        <v>330</v>
+      </c>
+      <c r="C112" s="134"/>
+      <c r="D112" s="134"/>
       <c r="E112" s="117" t="s">
         <v>222</v>
       </c>
       <c r="F112" s="118"/>
-      <c r="G112" s="133"/>
+      <c r="G112" s="133">
+        <v>3</v>
+      </c>
       <c r="H112" s="123"/>
-      <c r="I112" s="120"/>
+      <c r="I112" s="120" t="s">
+        <v>306</v>
+      </c>
     </row>
     <row r="113" ht="14.25" customHeight="1">
       <c r="B113" s="44" t="s">
-        <v>326</v>
+        <v>331</v>
       </c>
       <c r="C113" s="44"/>
       <c r="D113" s="44"/>
@@ -9064,7 +9453,7 @@
     </row>
     <row r="115">
       <c r="B115" s="132" t="s">
-        <v>327</v>
+        <v>332</v>
       </c>
       <c r="C115" s="132"/>
       <c r="D115" s="132"/>
@@ -9072,13 +9461,17 @@
         <v>222</v>
       </c>
       <c r="F115" s="118"/>
-      <c r="G115" s="133"/>
+      <c r="G115" s="133">
+        <v>1</v>
+      </c>
       <c r="H115" s="123"/>
-      <c r="I115" s="120"/>
+      <c r="I115" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="116">
       <c r="B116" s="126" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
       <c r="C116" s="126"/>
       <c r="D116" s="126"/>
@@ -9086,13 +9479,17 @@
         <v>222</v>
       </c>
       <c r="F116" s="118"/>
-      <c r="G116" s="133"/>
+      <c r="G116" s="133">
+        <v>1</v>
+      </c>
       <c r="H116" s="123"/>
-      <c r="I116" s="120"/>
+      <c r="I116" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="117">
       <c r="B117" s="126" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
       <c r="C117" s="126"/>
       <c r="D117" s="126"/>
@@ -9100,13 +9497,17 @@
         <v>222</v>
       </c>
       <c r="F117" s="118"/>
-      <c r="G117" s="133"/>
+      <c r="G117" s="133">
+        <v>1</v>
+      </c>
       <c r="H117" s="123"/>
-      <c r="I117" s="120"/>
+      <c r="I117" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="118">
       <c r="B118" s="126" t="s">
-        <v>330</v>
+        <v>335</v>
       </c>
       <c r="C118" s="126"/>
       <c r="D118" s="126"/>
@@ -9114,13 +9515,17 @@
         <v>222</v>
       </c>
       <c r="F118" s="118"/>
-      <c r="G118" s="133"/>
+      <c r="G118" s="133">
+        <v>1</v>
+      </c>
       <c r="H118" s="123"/>
-      <c r="I118" s="120"/>
+      <c r="I118" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="119">
       <c r="B119" s="126" t="s">
-        <v>331</v>
+        <v>336</v>
       </c>
       <c r="C119" s="126"/>
       <c r="D119" s="126"/>
@@ -9128,13 +9533,17 @@
         <v>222</v>
       </c>
       <c r="F119" s="118"/>
-      <c r="G119" s="133"/>
+      <c r="G119" s="133">
+        <v>1</v>
+      </c>
       <c r="H119" s="123"/>
-      <c r="I119" s="120"/>
+      <c r="I119" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="120">
       <c r="B120" s="126" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="C120" s="126"/>
       <c r="D120" s="126"/>
@@ -9142,13 +9551,17 @@
         <v>222</v>
       </c>
       <c r="F120" s="118"/>
-      <c r="G120" s="133"/>
+      <c r="G120" s="133">
+        <v>1</v>
+      </c>
       <c r="H120" s="123"/>
-      <c r="I120" s="120"/>
+      <c r="I120" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="121">
       <c r="B121" s="126" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="C121" s="126"/>
       <c r="D121" s="126"/>
@@ -9156,13 +9569,17 @@
         <v>222</v>
       </c>
       <c r="F121" s="118"/>
-      <c r="G121" s="133"/>
+      <c r="G121" s="133">
+        <v>1</v>
+      </c>
       <c r="H121" s="123"/>
-      <c r="I121" s="120"/>
+      <c r="I121" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="122">
       <c r="B122" s="126" t="s">
-        <v>334</v>
+        <v>339</v>
       </c>
       <c r="C122" s="126"/>
       <c r="D122" s="126"/>
@@ -9170,13 +9587,17 @@
         <v>222</v>
       </c>
       <c r="F122" s="118"/>
-      <c r="G122" s="133"/>
+      <c r="G122" s="133">
+        <v>1</v>
+      </c>
       <c r="H122" s="123"/>
-      <c r="I122" s="120"/>
+      <c r="I122" s="120" t="s">
+        <v>250</v>
+      </c>
     </row>
     <row r="123">
       <c r="B123" s="126" t="s">
-        <v>335</v>
+        <v>340</v>
       </c>
       <c r="C123" s="126"/>
       <c r="D123" s="126"/>
@@ -9184,13 +9605,17 @@
         <v>222</v>
       </c>
       <c r="F123" s="118"/>
-      <c r="G123" s="133"/>
+      <c r="G123" s="133">
+        <v>1</v>
+      </c>
       <c r="H123" s="123"/>
-      <c r="I123" s="120"/>
+      <c r="I123" s="120" t="s">
+        <v>250</v>
+      </c>
     </row>
     <row r="124">
       <c r="B124" s="126" t="s">
-        <v>336</v>
+        <v>341</v>
       </c>
       <c r="C124" s="126"/>
       <c r="D124" s="126"/>
@@ -9198,55 +9623,71 @@
         <v>222</v>
       </c>
       <c r="F124" s="118"/>
-      <c r="G124" s="133"/>
+      <c r="G124" s="133">
+        <v>1</v>
+      </c>
       <c r="H124" s="123"/>
-      <c r="I124" s="120"/>
+      <c r="I124" s="120" t="s">
+        <v>250</v>
+      </c>
     </row>
     <row r="125">
       <c r="B125" s="126" t="s">
-        <v>337</v>
+        <v>342</v>
       </c>
       <c r="C125" s="126"/>
       <c r="D125" s="126"/>
       <c r="E125" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F125" s="118"/>
-      <c r="G125" s="133"/>
+      <c r="G125" s="133">
+        <v>3</v>
+      </c>
       <c r="H125" s="123"/>
-      <c r="I125" s="120"/>
+      <c r="I125" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="126">
       <c r="B126" s="126" t="s">
-        <v>338</v>
+        <v>343</v>
       </c>
       <c r="C126" s="126"/>
       <c r="D126" s="126"/>
       <c r="E126" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F126" s="118"/>
-      <c r="G126" s="133"/>
+      <c r="G126" s="133">
+        <v>2</v>
+      </c>
       <c r="H126" s="123"/>
-      <c r="I126" s="120"/>
+      <c r="I126" s="120" t="s">
+        <v>250</v>
+      </c>
     </row>
     <row r="127">
       <c r="B127" s="126" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
       <c r="C127" s="126"/>
       <c r="D127" s="126"/>
       <c r="E127" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F127" s="118"/>
-      <c r="G127" s="133"/>
+      <c r="G127" s="133">
+        <v>2</v>
+      </c>
       <c r="H127" s="123"/>
-      <c r="I127" s="120"/>
+      <c r="I127" s="120" t="s">
+        <v>250</v>
+      </c>
     </row>
     <row r="128">
       <c r="B128" s="126" t="s">
-        <v>340</v>
+        <v>345</v>
       </c>
       <c r="C128" s="126"/>
       <c r="D128" s="126"/>
@@ -9254,13 +9695,17 @@
         <v>222</v>
       </c>
       <c r="F128" s="118"/>
-      <c r="G128" s="133"/>
+      <c r="G128" s="133">
+        <v>1</v>
+      </c>
       <c r="H128" s="123"/>
-      <c r="I128" s="120"/>
+      <c r="I128" s="120" t="s">
+        <v>250</v>
+      </c>
     </row>
     <row r="129">
       <c r="B129" s="126" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
       <c r="C129" s="126"/>
       <c r="D129" s="126"/>
@@ -9268,13 +9713,17 @@
         <v>222</v>
       </c>
       <c r="F129" s="118"/>
-      <c r="G129" s="133"/>
+      <c r="G129" s="133">
+        <v>1</v>
+      </c>
       <c r="H129" s="123"/>
-      <c r="I129" s="120"/>
+      <c r="I129" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="130">
       <c r="B130" s="126" t="s">
-        <v>342</v>
+        <v>347</v>
       </c>
       <c r="C130" s="126"/>
       <c r="D130" s="126"/>
@@ -9282,27 +9731,35 @@
         <v>222</v>
       </c>
       <c r="F130" s="118"/>
-      <c r="G130" s="133"/>
+      <c r="G130" s="133">
+        <v>1</v>
+      </c>
       <c r="H130" s="123"/>
-      <c r="I130" s="120"/>
+      <c r="I130" s="120" t="s">
+        <v>250</v>
+      </c>
     </row>
     <row r="131">
       <c r="B131" s="126" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
       <c r="C131" s="126"/>
       <c r="D131" s="126"/>
       <c r="E131" s="117" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F131" s="118"/>
-      <c r="G131" s="133"/>
+      <c r="G131" s="133">
+        <v>2</v>
+      </c>
       <c r="H131" s="123"/>
-      <c r="I131" s="120"/>
+      <c r="I131" s="120" t="s">
+        <v>250</v>
+      </c>
     </row>
     <row r="132" ht="14.25" customHeight="1">
       <c r="B132" s="44" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="C132" s="44"/>
       <c r="D132" s="44"/>
@@ -9331,18 +9788,22 @@
       <c r="I133" s="131"/>
     </row>
     <row r="134">
-      <c r="B134" s="136" t="s">
+      <c r="B134" s="135" t="s">
         <v>202</v>
       </c>
-      <c r="C134" s="136"/>
-      <c r="D134" s="136"/>
+      <c r="C134" s="135"/>
+      <c r="D134" s="135"/>
       <c r="E134" s="117" t="s">
         <v>222</v>
       </c>
       <c r="F134" s="118"/>
-      <c r="G134" s="133"/>
+      <c r="G134" s="133">
+        <v>4</v>
+      </c>
       <c r="H134" s="123"/>
-      <c r="I134" s="120"/>
+      <c r="I134" s="120" t="s">
+        <v>350</v>
+      </c>
     </row>
     <row r="135">
       <c r="B135" s="122" t="s">
@@ -9354,27 +9815,35 @@
         <v>222</v>
       </c>
       <c r="F135" s="118"/>
-      <c r="G135" s="133"/>
+      <c r="G135" s="133">
+        <v>4</v>
+      </c>
       <c r="H135" s="123"/>
-      <c r="I135" s="120"/>
+      <c r="I135" s="120" t="s">
+        <v>351</v>
+      </c>
     </row>
     <row r="136">
-      <c r="B136" s="137" t="s">
+      <c r="B136" s="136" t="s">
         <v>209</v>
       </c>
-      <c r="C136" s="138"/>
-      <c r="D136" s="139"/>
+      <c r="C136" s="137"/>
+      <c r="D136" s="138"/>
       <c r="E136" s="117" t="s">
         <v>222</v>
       </c>
       <c r="F136" s="118"/>
-      <c r="G136" s="133"/>
+      <c r="G136" s="133">
+        <v>2</v>
+      </c>
       <c r="H136" s="123"/>
-      <c r="I136" s="120"/>
+      <c r="I136" s="120" t="s">
+        <v>352</v>
+      </c>
     </row>
     <row r="137">
       <c r="B137" s="120" t="s">
-        <v>345</v>
+        <v>353</v>
       </c>
       <c r="C137" s="120"/>
       <c r="D137" s="120"/>
@@ -9382,139 +9851,179 @@
         <v>222</v>
       </c>
       <c r="F137" s="118"/>
-      <c r="G137" s="133"/>
+      <c r="G137" s="133">
+        <v>4</v>
+      </c>
       <c r="H137" s="123"/>
-      <c r="I137" s="120"/>
+      <c r="I137" s="120" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="138">
-      <c r="B138" s="137" t="s">
-        <v>346</v>
-      </c>
-      <c r="C138" s="138"/>
-      <c r="D138" s="139"/>
+      <c r="B138" s="136" t="s">
+        <v>354</v>
+      </c>
+      <c r="C138" s="137"/>
+      <c r="D138" s="138"/>
       <c r="E138" s="117" t="s">
         <v>222</v>
       </c>
       <c r="F138" s="118"/>
-      <c r="G138" s="133"/>
+      <c r="G138" s="133">
+        <v>4</v>
+      </c>
       <c r="H138" s="123"/>
-      <c r="I138" s="120"/>
+      <c r="I138" s="120" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="139">
-      <c r="B139" s="137" t="s">
-        <v>347</v>
-      </c>
-      <c r="C139" s="138"/>
-      <c r="D139" s="139"/>
+      <c r="B139" s="136" t="s">
+        <v>355</v>
+      </c>
+      <c r="C139" s="137"/>
+      <c r="D139" s="138"/>
       <c r="E139" s="117" t="s">
         <v>222</v>
       </c>
       <c r="F139" s="118"/>
-      <c r="G139" s="133"/>
+      <c r="G139" s="133">
+        <v>4</v>
+      </c>
       <c r="H139" s="123"/>
-      <c r="I139" s="120"/>
+      <c r="I139" s="120" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="140">
-      <c r="B140" s="137" t="s">
-        <v>348</v>
-      </c>
-      <c r="C140" s="138"/>
-      <c r="D140" s="139"/>
+      <c r="B140" s="136" t="s">
+        <v>356</v>
+      </c>
+      <c r="C140" s="137"/>
+      <c r="D140" s="138"/>
       <c r="E140" s="117" t="s">
         <v>222</v>
       </c>
       <c r="F140" s="118"/>
-      <c r="G140" s="133"/>
+      <c r="G140" s="133">
+        <v>4</v>
+      </c>
       <c r="H140" s="123"/>
-      <c r="I140" s="120"/>
+      <c r="I140" s="120" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="141">
-      <c r="B141" s="137" t="s">
-        <v>349</v>
-      </c>
-      <c r="C141" s="138"/>
-      <c r="D141" s="139"/>
+      <c r="B141" s="136" t="s">
+        <v>357</v>
+      </c>
+      <c r="C141" s="137"/>
+      <c r="D141" s="138"/>
       <c r="E141" s="117" t="s">
         <v>222</v>
       </c>
       <c r="F141" s="118"/>
-      <c r="G141" s="133"/>
+      <c r="G141" s="133">
+        <v>4</v>
+      </c>
       <c r="H141" s="123"/>
-      <c r="I141" s="120"/>
+      <c r="I141" s="120" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="142">
-      <c r="B142" s="137" t="s">
-        <v>350</v>
-      </c>
-      <c r="C142" s="138"/>
-      <c r="D142" s="139"/>
+      <c r="B142" s="136" t="s">
+        <v>358</v>
+      </c>
+      <c r="C142" s="137"/>
+      <c r="D142" s="138"/>
       <c r="E142" s="117" t="s">
         <v>222</v>
       </c>
       <c r="F142" s="118"/>
-      <c r="G142" s="133"/>
+      <c r="G142" s="133">
+        <v>4</v>
+      </c>
       <c r="H142" s="123"/>
-      <c r="I142" s="120"/>
+      <c r="I142" s="120" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="143">
-      <c r="B143" s="137" t="s">
-        <v>351</v>
-      </c>
-      <c r="C143" s="138"/>
-      <c r="D143" s="139"/>
+      <c r="B143" s="136" t="s">
+        <v>359</v>
+      </c>
+      <c r="C143" s="137"/>
+      <c r="D143" s="138"/>
       <c r="E143" s="117" t="s">
         <v>222</v>
       </c>
       <c r="F143" s="118"/>
-      <c r="G143" s="133"/>
+      <c r="G143" s="133">
+        <v>4</v>
+      </c>
       <c r="H143" s="123"/>
-      <c r="I143" s="120"/>
+      <c r="I143" s="120" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="144">
-      <c r="B144" s="137" t="s">
-        <v>352</v>
-      </c>
-      <c r="C144" s="138"/>
-      <c r="D144" s="139"/>
+      <c r="B144" s="136" t="s">
+        <v>360</v>
+      </c>
+      <c r="C144" s="137"/>
+      <c r="D144" s="138"/>
       <c r="E144" s="117" t="s">
         <v>222</v>
       </c>
       <c r="F144" s="118"/>
-      <c r="G144" s="133"/>
+      <c r="G144" s="133">
+        <v>4</v>
+      </c>
       <c r="H144" s="123"/>
-      <c r="I144" s="120"/>
+      <c r="I144" s="120" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="145">
-      <c r="B145" s="137" t="s">
-        <v>353</v>
-      </c>
-      <c r="C145" s="138"/>
-      <c r="D145" s="139"/>
+      <c r="B145" s="136" t="s">
+        <v>361</v>
+      </c>
+      <c r="C145" s="137"/>
+      <c r="D145" s="138"/>
       <c r="E145" s="117" t="s">
         <v>222</v>
       </c>
       <c r="F145" s="118"/>
-      <c r="G145" s="133"/>
+      <c r="G145" s="133">
+        <v>4</v>
+      </c>
       <c r="H145" s="123"/>
-      <c r="I145" s="120"/>
+      <c r="I145" s="120" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="146">
-      <c r="B146" s="137" t="s">
-        <v>354</v>
-      </c>
-      <c r="C146" s="138"/>
-      <c r="D146" s="139"/>
+      <c r="B146" s="136" t="s">
+        <v>362</v>
+      </c>
+      <c r="C146" s="137"/>
+      <c r="D146" s="138"/>
       <c r="E146" s="117" t="s">
         <v>222</v>
       </c>
       <c r="F146" s="118"/>
-      <c r="G146" s="133"/>
+      <c r="G146" s="133">
+        <v>4</v>
+      </c>
       <c r="H146" s="123"/>
-      <c r="I146" s="120"/>
+      <c r="I146" s="120" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="147">
       <c r="B147" s="120" t="s">
-        <v>355</v>
+        <v>363</v>
       </c>
       <c r="C147" s="120"/>
       <c r="D147" s="120"/>
@@ -9522,13 +10031,17 @@
         <v>222</v>
       </c>
       <c r="F147" s="118"/>
-      <c r="G147" s="133"/>
+      <c r="G147" s="133">
+        <v>3</v>
+      </c>
       <c r="H147" s="123"/>
-      <c r="I147" s="120"/>
+      <c r="I147" s="120" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="148">
       <c r="B148" s="120" t="s">
-        <v>356</v>
+        <v>364</v>
       </c>
       <c r="C148" s="120"/>
       <c r="D148" s="120"/>
@@ -9536,13 +10049,17 @@
         <v>222</v>
       </c>
       <c r="F148" s="118"/>
-      <c r="G148" s="133"/>
+      <c r="G148" s="133">
+        <v>3</v>
+      </c>
       <c r="H148" s="123"/>
-      <c r="I148" s="120"/>
+      <c r="I148" s="120" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="149">
       <c r="B149" s="120" t="s">
-        <v>357</v>
+        <v>365</v>
       </c>
       <c r="C149" s="120"/>
       <c r="D149" s="120"/>
@@ -9550,13 +10067,17 @@
         <v>222</v>
       </c>
       <c r="F149" s="118"/>
-      <c r="G149" s="133"/>
+      <c r="G149" s="133">
+        <v>2</v>
+      </c>
       <c r="H149" s="123"/>
-      <c r="I149" s="120"/>
+      <c r="I149" s="120" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="150">
       <c r="B150" s="120" t="s">
-        <v>358</v>
+        <v>366</v>
       </c>
       <c r="C150" s="120"/>
       <c r="D150" s="120"/>
@@ -9564,139 +10085,179 @@
         <v>222</v>
       </c>
       <c r="F150" s="118"/>
-      <c r="G150" s="133"/>
+      <c r="G150" s="133">
+        <v>3</v>
+      </c>
       <c r="H150" s="123"/>
-      <c r="I150" s="120"/>
+      <c r="I150" s="120" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="151">
       <c r="B151" s="120" t="s">
-        <v>359</v>
+        <v>367</v>
       </c>
       <c r="C151" s="120"/>
       <c r="D151" s="120"/>
       <c r="E151" s="117" t="s">
+        <v>368</v>
+      </c>
+      <c r="F151" s="118"/>
+      <c r="G151" s="133">
+        <v>2</v>
+      </c>
+      <c r="H151" s="123"/>
+      <c r="I151" s="120" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="B152" s="136" t="s">
+        <v>369</v>
+      </c>
+      <c r="C152" s="137"/>
+      <c r="D152" s="138"/>
+      <c r="E152" s="117" t="s">
+        <v>368</v>
+      </c>
+      <c r="F152" s="118"/>
+      <c r="G152" s="133">
+        <v>2</v>
+      </c>
+      <c r="H152" s="123"/>
+      <c r="I152" s="120" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="B153" s="136" t="s">
+        <v>370</v>
+      </c>
+      <c r="C153" s="137"/>
+      <c r="D153" s="138"/>
+      <c r="E153" s="117" t="s">
+        <v>368</v>
+      </c>
+      <c r="F153" s="118"/>
+      <c r="G153" s="133">
+        <v>2</v>
+      </c>
+      <c r="H153" s="123"/>
+      <c r="I153" s="120" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="B154" s="136" t="s">
+        <v>371</v>
+      </c>
+      <c r="C154" s="137"/>
+      <c r="D154" s="138"/>
+      <c r="E154" s="117" t="s">
+        <v>368</v>
+      </c>
+      <c r="F154" s="118"/>
+      <c r="G154" s="133">
+        <v>2</v>
+      </c>
+      <c r="H154" s="123"/>
+      <c r="I154" s="120" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="B155" s="136" t="s">
+        <v>372</v>
+      </c>
+      <c r="C155" s="137"/>
+      <c r="D155" s="138"/>
+      <c r="E155" s="117" t="s">
+        <v>368</v>
+      </c>
+      <c r="F155" s="118"/>
+      <c r="G155" s="133">
+        <v>2</v>
+      </c>
+      <c r="H155" s="123"/>
+      <c r="I155" s="120" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="B156" s="136" t="s">
+        <v>373</v>
+      </c>
+      <c r="C156" s="137"/>
+      <c r="D156" s="138"/>
+      <c r="E156" s="117" t="s">
         <v>222</v>
       </c>
-      <c r="F151" s="118"/>
-      <c r="G151" s="133"/>
-      <c r="H151" s="123"/>
-      <c r="I151" s="120"/>
-    </row>
-    <row r="152">
-      <c r="B152" s="120" t="s">
-        <v>360</v>
-      </c>
-      <c r="C152" s="120"/>
-      <c r="D152" s="120"/>
-      <c r="E152" s="117" t="s">
+      <c r="F156" s="118"/>
+      <c r="G156" s="133">
+        <v>2</v>
+      </c>
+      <c r="H156" s="123"/>
+      <c r="I156" s="120" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="B157" s="136" t="s">
+        <v>374</v>
+      </c>
+      <c r="C157" s="137"/>
+      <c r="D157" s="138"/>
+      <c r="E157" s="117" t="s">
         <v>222</v>
       </c>
-      <c r="F152" s="118"/>
-      <c r="G152" s="133"/>
-      <c r="H152" s="123"/>
-      <c r="I152" s="120"/>
-    </row>
-    <row r="153">
-      <c r="B153" s="120" t="s">
-        <v>361</v>
-      </c>
-      <c r="C153" s="120"/>
-      <c r="D153" s="120"/>
-      <c r="E153" s="117" t="s">
-        <v>362</v>
-      </c>
-      <c r="F153" s="118"/>
-      <c r="G153" s="133"/>
-      <c r="H153" s="123"/>
-      <c r="I153" s="120"/>
-    </row>
-    <row r="154">
-      <c r="B154" s="137" t="s">
-        <v>363</v>
-      </c>
-      <c r="C154" s="138"/>
-      <c r="D154" s="139"/>
-      <c r="E154" s="117" t="s">
-        <v>362</v>
-      </c>
-      <c r="F154" s="118"/>
-      <c r="G154" s="133"/>
-      <c r="H154" s="123"/>
-      <c r="I154" s="120"/>
-    </row>
-    <row r="155">
-      <c r="B155" s="137" t="s">
-        <v>364</v>
-      </c>
-      <c r="C155" s="138"/>
-      <c r="D155" s="139"/>
-      <c r="E155" s="117" t="s">
-        <v>362</v>
-      </c>
-      <c r="F155" s="118"/>
-      <c r="G155" s="133"/>
-      <c r="H155" s="123"/>
-      <c r="I155" s="120"/>
-    </row>
-    <row r="156">
-      <c r="B156" s="137" t="s">
-        <v>365</v>
-      </c>
-      <c r="C156" s="138"/>
-      <c r="D156" s="139"/>
-      <c r="E156" s="117" t="s">
-        <v>362</v>
-      </c>
-      <c r="F156" s="118"/>
-      <c r="G156" s="133"/>
-      <c r="H156" s="123"/>
-      <c r="I156" s="120"/>
-    </row>
-    <row r="157">
-      <c r="B157" s="137" t="s">
-        <v>366</v>
-      </c>
-      <c r="C157" s="138"/>
-      <c r="D157" s="139"/>
-      <c r="E157" s="117" t="s">
-        <v>362</v>
-      </c>
       <c r="F157" s="118"/>
-      <c r="G157" s="133"/>
+      <c r="G157" s="133">
+        <v>2</v>
+      </c>
       <c r="H157" s="123"/>
-      <c r="I157" s="120"/>
+      <c r="I157" s="120" t="s">
+        <v>352</v>
+      </c>
     </row>
     <row r="158">
-      <c r="B158" s="137" t="s">
-        <v>367</v>
-      </c>
-      <c r="C158" s="138"/>
-      <c r="D158" s="139"/>
+      <c r="B158" s="126" t="s">
+        <v>375</v>
+      </c>
+      <c r="C158" s="126"/>
+      <c r="D158" s="126"/>
       <c r="E158" s="117" t="s">
         <v>222</v>
       </c>
       <c r="F158" s="118"/>
-      <c r="G158" s="133"/>
+      <c r="G158" s="133">
+        <v>2</v>
+      </c>
       <c r="H158" s="123"/>
-      <c r="I158" s="120"/>
+      <c r="I158" s="120" t="s">
+        <v>352</v>
+      </c>
     </row>
     <row r="159">
-      <c r="B159" s="137" t="s">
-        <v>368</v>
-      </c>
-      <c r="C159" s="138"/>
-      <c r="D159" s="139"/>
+      <c r="B159" s="126" t="s">
+        <v>376</v>
+      </c>
+      <c r="C159" s="126"/>
+      <c r="D159" s="126"/>
       <c r="E159" s="117" t="s">
         <v>222</v>
       </c>
       <c r="F159" s="118"/>
-      <c r="G159" s="133"/>
+      <c r="G159" s="133">
+        <v>2</v>
+      </c>
       <c r="H159" s="123"/>
-      <c r="I159" s="120"/>
+      <c r="I159" s="120" t="s">
+        <v>352</v>
+      </c>
     </row>
     <row r="160">
       <c r="B160" s="126" t="s">
-        <v>369</v>
+        <v>377</v>
       </c>
       <c r="C160" s="126"/>
       <c r="D160" s="126"/>
@@ -9704,13 +10265,17 @@
         <v>222</v>
       </c>
       <c r="F160" s="118"/>
-      <c r="G160" s="133"/>
+      <c r="G160" s="133">
+        <v>3</v>
+      </c>
       <c r="H160" s="123"/>
-      <c r="I160" s="120"/>
+      <c r="I160" s="120" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="161">
       <c r="B161" s="126" t="s">
-        <v>370</v>
+        <v>378</v>
       </c>
       <c r="C161" s="126"/>
       <c r="D161" s="126"/>
@@ -9718,13 +10283,17 @@
         <v>222</v>
       </c>
       <c r="F161" s="118"/>
-      <c r="G161" s="133"/>
+      <c r="G161" s="133">
+        <v>2</v>
+      </c>
       <c r="H161" s="123"/>
-      <c r="I161" s="120"/>
+      <c r="I161" s="120" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="162">
       <c r="B162" s="126" t="s">
-        <v>371</v>
+        <v>379</v>
       </c>
       <c r="C162" s="126"/>
       <c r="D162" s="126"/>
@@ -9732,13 +10301,17 @@
         <v>222</v>
       </c>
       <c r="F162" s="118"/>
-      <c r="G162" s="133"/>
+      <c r="G162" s="133">
+        <v>2</v>
+      </c>
       <c r="H162" s="123"/>
-      <c r="I162" s="120"/>
+      <c r="I162" s="120" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="163">
       <c r="B163" s="126" t="s">
-        <v>372</v>
+        <v>380</v>
       </c>
       <c r="C163" s="126"/>
       <c r="D163" s="126"/>
@@ -9746,13 +10319,17 @@
         <v>222</v>
       </c>
       <c r="F163" s="118"/>
-      <c r="G163" s="133"/>
+      <c r="G163" s="133">
+        <v>2</v>
+      </c>
       <c r="H163" s="123"/>
-      <c r="I163" s="120"/>
+      <c r="I163" s="120" t="s">
+        <v>252</v>
+      </c>
     </row>
     <row r="164">
       <c r="B164" s="126" t="s">
-        <v>373</v>
+        <v>381</v>
       </c>
       <c r="C164" s="126"/>
       <c r="D164" s="126"/>
@@ -9760,13 +10337,17 @@
         <v>222</v>
       </c>
       <c r="F164" s="118"/>
-      <c r="G164" s="133"/>
+      <c r="G164" s="133">
+        <v>2</v>
+      </c>
       <c r="H164" s="123"/>
-      <c r="I164" s="120"/>
+      <c r="I164" s="120" t="s">
+        <v>252</v>
+      </c>
     </row>
     <row r="165">
       <c r="B165" s="126" t="s">
-        <v>374</v>
+        <v>382</v>
       </c>
       <c r="C165" s="126"/>
       <c r="D165" s="126"/>
@@ -9774,13 +10355,17 @@
         <v>222</v>
       </c>
       <c r="F165" s="118"/>
-      <c r="G165" s="133"/>
+      <c r="G165" s="133">
+        <v>2</v>
+      </c>
       <c r="H165" s="123"/>
-      <c r="I165" s="120"/>
+      <c r="I165" s="120" t="s">
+        <v>252</v>
+      </c>
     </row>
     <row r="166">
       <c r="B166" s="126" t="s">
-        <v>375</v>
+        <v>383</v>
       </c>
       <c r="C166" s="126"/>
       <c r="D166" s="126"/>
@@ -9788,13 +10373,17 @@
         <v>222</v>
       </c>
       <c r="F166" s="118"/>
-      <c r="G166" s="133"/>
+      <c r="G166" s="133">
+        <v>2</v>
+      </c>
       <c r="H166" s="123"/>
-      <c r="I166" s="120"/>
+      <c r="I166" s="120" t="s">
+        <v>252</v>
+      </c>
     </row>
     <row r="167">
       <c r="B167" s="126" t="s">
-        <v>376</v>
+        <v>384</v>
       </c>
       <c r="C167" s="126"/>
       <c r="D167" s="126"/>
@@ -9802,13 +10391,17 @@
         <v>222</v>
       </c>
       <c r="F167" s="118"/>
-      <c r="G167" s="133"/>
+      <c r="G167" s="133">
+        <v>2</v>
+      </c>
       <c r="H167" s="123"/>
-      <c r="I167" s="120"/>
+      <c r="I167" s="120" t="s">
+        <v>252</v>
+      </c>
     </row>
     <row r="168">
       <c r="B168" s="126" t="s">
-        <v>377</v>
+        <v>385</v>
       </c>
       <c r="C168" s="126"/>
       <c r="D168" s="126"/>
@@ -9816,13 +10409,17 @@
         <v>222</v>
       </c>
       <c r="F168" s="118"/>
-      <c r="G168" s="133"/>
+      <c r="G168" s="133">
+        <v>2</v>
+      </c>
       <c r="H168" s="123"/>
-      <c r="I168" s="120"/>
+      <c r="I168" s="120" t="s">
+        <v>252</v>
+      </c>
     </row>
     <row r="169">
       <c r="B169" s="126" t="s">
-        <v>378</v>
+        <v>386</v>
       </c>
       <c r="C169" s="126"/>
       <c r="D169" s="126"/>
@@ -9830,97 +10427,87 @@
         <v>222</v>
       </c>
       <c r="F169" s="118"/>
-      <c r="G169" s="133"/>
+      <c r="G169" s="133">
+        <v>2</v>
+      </c>
       <c r="H169" s="123"/>
-      <c r="I169" s="120"/>
+      <c r="I169" s="120" t="s">
+        <v>252</v>
+      </c>
     </row>
     <row r="170">
-      <c r="B170" s="126" t="s">
-        <v>379</v>
-      </c>
-      <c r="C170" s="126"/>
-      <c r="D170" s="126"/>
-      <c r="E170" s="117" t="s">
-        <v>222</v>
-      </c>
-      <c r="F170" s="118"/>
-      <c r="G170" s="133"/>
-      <c r="H170" s="123"/>
-      <c r="I170" s="120"/>
+      <c r="E170" s="2"/>
+      <c r="F170" s="4"/>
+      <c r="G170" s="109"/>
+      <c r="H170" s="6"/>
+      <c r="I170" s="110"/>
     </row>
     <row r="171">
-      <c r="B171" s="126" t="s">
-        <v>380</v>
-      </c>
-      <c r="C171" s="126"/>
-      <c r="D171" s="126"/>
-      <c r="E171" s="117" t="s">
-        <v>222</v>
-      </c>
-      <c r="F171" s="118"/>
-      <c r="G171" s="133"/>
-      <c r="H171" s="123"/>
-      <c r="I171" s="120"/>
+      <c r="D171" s="103"/>
+      <c r="E171" s="139"/>
+      <c r="F171" s="140"/>
+      <c r="G171" s="141"/>
+      <c r="H171" s="140"/>
+      <c r="I171" s="140"/>
     </row>
     <row r="172">
-      <c r="E172" s="2"/>
-      <c r="F172" s="4"/>
-      <c r="G172" s="109"/>
-      <c r="H172" s="6"/>
-      <c r="I172" s="110"/>
+      <c r="D172" s="103"/>
+      <c r="E172" s="103"/>
+      <c r="F172" s="103"/>
+      <c r="H172" s="142"/>
     </row>
     <row r="173">
       <c r="D173" s="103"/>
-      <c r="E173" s="140"/>
-      <c r="F173" s="141"/>
-      <c r="G173" s="142"/>
-      <c r="H173" s="141"/>
-      <c r="I173" s="141"/>
+      <c r="E173" s="103"/>
+      <c r="F173" s="103"/>
+      <c r="H173" s="142"/>
     </row>
     <row r="174">
       <c r="D174" s="103"/>
       <c r="E174" s="103"/>
       <c r="F174" s="103"/>
-      <c r="H174" s="143"/>
+      <c r="H174" s="142"/>
     </row>
     <row r="175">
       <c r="D175" s="103"/>
       <c r="E175" s="103"/>
       <c r="F175" s="103"/>
-      <c r="H175" s="143"/>
+      <c r="H175" s="142"/>
     </row>
     <row r="176">
       <c r="D176" s="103"/>
-      <c r="E176" s="103"/>
-      <c r="F176" s="103"/>
-      <c r="H176" s="143"/>
+      <c r="E176" s="139"/>
+      <c r="F176" s="140"/>
+      <c r="G176" s="143"/>
+      <c r="H176" s="141"/>
     </row>
     <row r="177">
       <c r="D177" s="103"/>
-      <c r="E177" s="103"/>
-      <c r="F177" s="103"/>
-      <c r="H177" s="143"/>
+      <c r="H177" s="142"/>
     </row>
     <row r="178">
+      <c r="B178" s="1" t="s">
+        <v>2</v>
+      </c>
       <c r="D178" s="103"/>
-      <c r="E178" s="140"/>
-      <c r="F178" s="141"/>
-      <c r="G178" s="144"/>
-      <c r="H178" s="142"/>
+      <c r="E178" s="139"/>
+      <c r="F178" s="140"/>
+      <c r="G178" s="143"/>
+      <c r="H178" s="141"/>
     </row>
     <row r="179">
-      <c r="D179" s="103"/>
-      <c r="H179" s="143"/>
+      <c r="E179" s="2"/>
+      <c r="F179" s="4"/>
+      <c r="G179" s="109"/>
+      <c r="H179" s="6"/>
+      <c r="I179" s="110"/>
     </row>
     <row r="180">
-      <c r="B180" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D180" s="103"/>
-      <c r="E180" s="140"/>
-      <c r="F180" s="141"/>
-      <c r="G180" s="144"/>
-      <c r="H180" s="142"/>
+      <c r="E180" s="2"/>
+      <c r="F180" s="4"/>
+      <c r="G180" s="109"/>
+      <c r="H180" s="6"/>
+      <c r="I180" s="110"/>
     </row>
     <row r="181">
       <c r="E181" s="2"/>
@@ -10195,19 +10782,21 @@
       <c r="H219" s="6"/>
       <c r="I219" s="110"/>
     </row>
-    <row r="220">
+    <row r="220" s="1" customFormat="1">
       <c r="E220" s="2"/>
       <c r="F220" s="4"/>
       <c r="G220" s="109"/>
       <c r="H220" s="6"/>
       <c r="I220" s="110"/>
-    </row>
-    <row r="221">
+      <c r="W220" s="103"/>
+    </row>
+    <row r="221" s="1" customFormat="1">
       <c r="E221" s="2"/>
       <c r="F221" s="4"/>
       <c r="G221" s="109"/>
       <c r="H221" s="6"/>
       <c r="I221" s="110"/>
+      <c r="W221" s="103"/>
     </row>
     <row r="222" s="1" customFormat="1">
       <c r="E222" s="2"/>
@@ -11225,21 +11814,15 @@
       <c r="I348" s="110"/>
       <c r="W348" s="103"/>
     </row>
-    <row r="349" s="1" customFormat="1">
+    <row r="349">
       <c r="E349" s="2"/>
       <c r="F349" s="4"/>
       <c r="G349" s="109"/>
-      <c r="H349" s="6"/>
-      <c r="I349" s="110"/>
-      <c r="W349" s="103"/>
-    </row>
-    <row r="350" s="1" customFormat="1">
+    </row>
+    <row r="350">
       <c r="E350" s="2"/>
       <c r="F350" s="4"/>
       <c r="G350" s="109"/>
-      <c r="H350" s="6"/>
-      <c r="I350" s="110"/>
-      <c r="W350" s="103"/>
     </row>
     <row r="351">
       <c r="E351" s="2"/>
@@ -12321,18 +12904,8 @@
       <c r="F566" s="4"/>
       <c r="G566" s="109"/>
     </row>
-    <row r="567">
-      <c r="E567" s="2"/>
-      <c r="F567" s="4"/>
-      <c r="G567" s="109"/>
-    </row>
-    <row r="568">
-      <c r="E568" s="2"/>
-      <c r="F568" s="4"/>
-      <c r="G568" s="109"/>
-    </row>
   </sheetData>
-  <mergeCells count="68">
+  <mergeCells count="66">
     <mergeCell ref="B5:D6"/>
     <mergeCell ref="E5:G5"/>
     <mergeCell ref="I5:I6"/>
@@ -12397,10 +12970,8 @@
     <mergeCell ref="B149:D149"/>
     <mergeCell ref="B150:D150"/>
     <mergeCell ref="B151:D151"/>
-    <mergeCell ref="B152:D152"/>
-    <mergeCell ref="B153:D153"/>
-    <mergeCell ref="B160:D160"/>
-    <mergeCell ref="B171:D171"/>
+    <mergeCell ref="B158:D158"/>
+    <mergeCell ref="B169:D169"/>
   </mergeCells>
   <printOptions headings="0" gridLines="0" horizontalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.64999999999999991" header="0.25" footer="0.25"/>

</xml_diff>

<commit_message>
feat(accounting,events,hub): GL anomaly detection, equipment rental pricing, connection pooling
- Accounting: Add GL anomaly review system with nightly rules engine + Claude AI
  analysis, statistical baselines, flag lifecycle, and dedicated UI page
- Events: Convert equipment/rentals from free-text to structured line items with
  name, quantity, and price that factor into financial totals and PDFs
- Events: Fix calendar item CalDAV sync venue lookup for location-to-venue mapping
- Hub: Centralize cross-DB connection management with pooling (eliminate 20+ inline
  create_engine calls), add get_inventory_engine() shared function
- Consolidate food-safety and maintenance docker-compose into root compose file
- Update CLAUDE.md and README.md with new feature documentation

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/files/storage/user_6/Corporate Files/SW Grill Boca Files/General Forms/Kitchen and Bar Order Sheet.xlsx
+++ b/files/storage/user_6/Corporate Files/SW Grill Boca Files/General Forms/Kitchen and Bar Order Sheet.xlsx
@@ -12,7 +12,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">FOOD!$C$1:$I$222</definedName>
     <definedName name="Print_Titles" localSheetId="0">FOOD!$1:$6</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">BAR!$B$1:$I$178</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">BAR!$B$1:$I$172</definedName>
     <definedName name="Print_Titles" localSheetId="1">BAR!$1:$6</definedName>
   </definedNames>
   <calcPr iterateDelta="0.0001"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="387" uniqueCount="387">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="381" uniqueCount="381">
   <si>
     <t xml:space="preserve">SW Grill</t>
   </si>
@@ -826,9 +826,6 @@
     <t xml:space="preserve">Angels Envy</t>
   </si>
   <si>
-    <t>Templeton</t>
-  </si>
-  <si>
     <t>Dewars</t>
   </si>
   <si>
@@ -838,9 +835,6 @@
     <t xml:space="preserve">Johnnie Walker Black</t>
   </si>
   <si>
-    <t>Oban</t>
-  </si>
-  <si>
     <t>Macallen</t>
   </si>
   <si>
@@ -1054,12 +1048,6 @@
     <t xml:space="preserve">Veuve Clicquot</t>
   </si>
   <si>
-    <t xml:space="preserve">Luxe Belaire White</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Luxe Belaire Rose</t>
-  </si>
-  <si>
     <t xml:space="preserve">Santa Margarita Prosecco</t>
   </si>
   <si>
@@ -1069,9 +1057,6 @@
     <t xml:space="preserve">Capriccio Sangria</t>
   </si>
   <si>
-    <t xml:space="preserve">Blue Mascato</t>
-  </si>
-  <si>
     <t>NAB</t>
   </si>
   <si>
@@ -1133,9 +1118,6 @@
   </si>
   <si>
     <t xml:space="preserve">BIB Diet Coke</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BIB Coke Zero</t>
   </si>
   <si>
     <t xml:space="preserve">BIB Sprite</t>
@@ -8309,7 +8291,9 @@
         <v>1</v>
       </c>
       <c r="H49" s="123"/>
-      <c r="I49" s="120"/>
+      <c r="I49" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="50">
       <c r="B50" s="128" t="s">
@@ -8340,7 +8324,7 @@
       </c>
       <c r="F51" s="118"/>
       <c r="G51" s="119">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H51" s="123"/>
       <c r="I51" s="120" t="s">
@@ -8362,7 +8346,7 @@
       </c>
       <c r="H52" s="123"/>
       <c r="I52" s="120" t="s">
-        <v>224</v>
+        <v>250</v>
       </c>
     </row>
     <row r="53">
@@ -8380,26 +8364,20 @@
       </c>
       <c r="H53" s="123"/>
       <c r="I53" s="120" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="B54" s="128" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="54" ht="16.5">
+      <c r="B54" s="129" t="s">
         <v>272</v>
       </c>
-      <c r="C54" s="128"/>
+      <c r="C54" s="129"/>
       <c r="D54" s="128"/>
-      <c r="E54" s="117" t="s">
-        <v>227</v>
-      </c>
+      <c r="E54" s="117"/>
       <c r="F54" s="118"/>
-      <c r="G54" s="119">
-        <v>2</v>
-      </c>
+      <c r="G54" s="119"/>
       <c r="H54" s="123"/>
-      <c r="I54" s="120" t="s">
-        <v>250</v>
-      </c>
+      <c r="I54" s="120"/>
     </row>
     <row r="55">
       <c r="B55" s="128" t="s">
@@ -8412,24 +8390,30 @@
       </c>
       <c r="F55" s="118"/>
       <c r="G55" s="119">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H55" s="123"/>
       <c r="I55" s="120" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="56" ht="16.5">
-      <c r="B56" s="129" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" s="128" t="s">
         <v>274</v>
       </c>
-      <c r="C56" s="129"/>
+      <c r="C56" s="128"/>
       <c r="D56" s="128"/>
-      <c r="E56" s="117"/>
+      <c r="E56" s="117" t="s">
+        <v>227</v>
+      </c>
       <c r="F56" s="118"/>
-      <c r="G56" s="119"/>
+      <c r="G56" s="119">
+        <v>4</v>
+      </c>
       <c r="H56" s="123"/>
-      <c r="I56" s="120"/>
+      <c r="I56" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="57">
       <c r="B57" s="128" t="s">
@@ -8442,11 +8426,11 @@
       </c>
       <c r="F57" s="118"/>
       <c r="G57" s="119">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H57" s="123"/>
       <c r="I57" s="120" t="s">
-        <v>224</v>
+        <v>250</v>
       </c>
     </row>
     <row r="58">
@@ -8460,11 +8444,11 @@
       </c>
       <c r="F58" s="118"/>
       <c r="G58" s="119">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H58" s="123"/>
       <c r="I58" s="120" t="s">
-        <v>224</v>
+        <v>250</v>
       </c>
     </row>
     <row r="59">
@@ -8485,23 +8469,17 @@
         <v>250</v>
       </c>
     </row>
-    <row r="60">
-      <c r="B60" s="128" t="s">
+    <row r="60" ht="16.5">
+      <c r="B60" s="129" t="s">
         <v>278</v>
       </c>
       <c r="C60" s="128"/>
       <c r="D60" s="128"/>
-      <c r="E60" s="117" t="s">
-        <v>227</v>
-      </c>
+      <c r="E60" s="117"/>
       <c r="F60" s="118"/>
-      <c r="G60" s="119">
-        <v>1</v>
-      </c>
+      <c r="G60" s="119"/>
       <c r="H60" s="123"/>
-      <c r="I60" s="120" t="s">
-        <v>250</v>
-      </c>
+      <c r="I60" s="120"/>
     </row>
     <row r="61">
       <c r="B61" s="128" t="s">
@@ -8518,20 +8496,26 @@
       </c>
       <c r="H61" s="123"/>
       <c r="I61" s="120" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="62" ht="16.5">
-      <c r="B62" s="129" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" s="128" t="s">
         <v>280</v>
       </c>
       <c r="C62" s="128"/>
       <c r="D62" s="128"/>
-      <c r="E62" s="117"/>
+      <c r="E62" s="117" t="s">
+        <v>227</v>
+      </c>
       <c r="F62" s="118"/>
-      <c r="G62" s="119"/>
+      <c r="G62" s="119">
+        <v>2</v>
+      </c>
       <c r="H62" s="123"/>
-      <c r="I62" s="120"/>
+      <c r="I62" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="63">
       <c r="B63" s="128" t="s">
@@ -8544,7 +8528,7 @@
       </c>
       <c r="F63" s="118"/>
       <c r="G63" s="119">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H63" s="123"/>
       <c r="I63" s="120" t="s">
@@ -8562,7 +8546,7 @@
       </c>
       <c r="F64" s="118"/>
       <c r="G64" s="119">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H64" s="123"/>
       <c r="I64" s="120" t="s">
@@ -8580,7 +8564,7 @@
       </c>
       <c r="F65" s="118"/>
       <c r="G65" s="119">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H65" s="123"/>
       <c r="I65" s="120" t="s">
@@ -8598,7 +8582,7 @@
       </c>
       <c r="F66" s="118"/>
       <c r="G66" s="119">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H66" s="123"/>
       <c r="I66" s="120" t="s">
@@ -8616,11 +8600,11 @@
       </c>
       <c r="F67" s="118"/>
       <c r="G67" s="119">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H67" s="123"/>
       <c r="I67" s="120" t="s">
-        <v>224</v>
+        <v>252</v>
       </c>
     </row>
     <row r="68">
@@ -8634,7 +8618,7 @@
       </c>
       <c r="F68" s="118"/>
       <c r="G68" s="119">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H68" s="123"/>
       <c r="I68" s="120" t="s">
@@ -8648,15 +8632,15 @@
       <c r="C69" s="128"/>
       <c r="D69" s="128"/>
       <c r="E69" s="117" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="F69" s="118"/>
       <c r="G69" s="119">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H69" s="123"/>
       <c r="I69" s="120" t="s">
-        <v>252</v>
+        <v>224</v>
       </c>
     </row>
     <row r="70">
@@ -8666,7 +8650,7 @@
       <c r="C70" s="128"/>
       <c r="D70" s="128"/>
       <c r="E70" s="117" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="F70" s="118"/>
       <c r="G70" s="119">
@@ -8692,7 +8676,7 @@
       </c>
       <c r="H71" s="123"/>
       <c r="I71" s="120" t="s">
-        <v>224</v>
+        <v>250</v>
       </c>
     </row>
     <row r="72">
@@ -8702,7 +8686,7 @@
       <c r="C72" s="128"/>
       <c r="D72" s="128"/>
       <c r="E72" s="117" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="F72" s="118"/>
       <c r="G72" s="119">
@@ -8720,7 +8704,7 @@
       <c r="C73" s="128"/>
       <c r="D73" s="128"/>
       <c r="E73" s="117" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="F73" s="118"/>
       <c r="G73" s="119">
@@ -8728,7 +8712,7 @@
       </c>
       <c r="H73" s="123"/>
       <c r="I73" s="120" t="s">
-        <v>250</v>
+        <v>224</v>
       </c>
     </row>
     <row r="74">
@@ -8814,7 +8798,7 @@
       </c>
       <c r="F78" s="118"/>
       <c r="G78" s="119">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H78" s="123"/>
       <c r="I78" s="120" t="s">
@@ -8828,7 +8812,7 @@
       <c r="C79" s="128"/>
       <c r="D79" s="128"/>
       <c r="E79" s="117" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="F79" s="118"/>
       <c r="G79" s="119">
@@ -8850,7 +8834,7 @@
       </c>
       <c r="F80" s="118"/>
       <c r="G80" s="119">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H80" s="123"/>
       <c r="I80" s="120" t="s">
@@ -8864,7 +8848,7 @@
       <c r="C81" s="128"/>
       <c r="D81" s="128"/>
       <c r="E81" s="117" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="F81" s="118"/>
       <c r="G81" s="119">
@@ -8894,13 +8878,13 @@
       </c>
     </row>
     <row r="83">
-      <c r="B83" s="128" t="s">
+      <c r="B83" s="130" t="s">
         <v>301</v>
       </c>
-      <c r="C83" s="128"/>
-      <c r="D83" s="128"/>
+      <c r="C83" s="130"/>
+      <c r="D83" s="130"/>
       <c r="E83" s="117" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="F83" s="118"/>
       <c r="G83" s="119">
@@ -8911,124 +8895,124 @@
         <v>224</v>
       </c>
     </row>
-    <row r="84">
-      <c r="B84" s="128" t="s">
+    <row r="84" ht="15" customHeight="1">
+      <c r="B84" s="44" t="s">
         <v>302</v>
       </c>
-      <c r="C84" s="128"/>
-      <c r="D84" s="128"/>
-      <c r="E84" s="117" t="s">
-        <v>227</v>
-      </c>
-      <c r="F84" s="118"/>
-      <c r="G84" s="119">
-        <v>1</v>
-      </c>
-      <c r="H84" s="123"/>
-      <c r="I84" s="120" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="85">
-      <c r="B85" s="130" t="s">
+      <c r="C84" s="44"/>
+      <c r="D84" s="44"/>
+      <c r="E84" s="45"/>
+      <c r="F84" s="45"/>
+      <c r="G84" s="45"/>
+      <c r="H84" s="46"/>
+      <c r="I84" s="131" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="85" ht="15" customHeight="1">
+      <c r="B85" s="44"/>
+      <c r="C85" s="44"/>
+      <c r="D85" s="44"/>
+      <c r="E85" s="49" t="s">
+        <v>5</v>
+      </c>
+      <c r="F85" s="50" t="s">
+        <v>6</v>
+      </c>
+      <c r="G85" s="51" t="s">
+        <v>7</v>
+      </c>
+      <c r="H85" s="52"/>
+      <c r="I85" s="131"/>
+    </row>
+    <row r="86">
+      <c r="B86" s="132" t="s">
         <v>303</v>
       </c>
-      <c r="C85" s="130"/>
-      <c r="D85" s="130"/>
-      <c r="E85" s="117" t="s">
+      <c r="C86" s="132"/>
+      <c r="D86" s="132"/>
+      <c r="E86" s="117" t="s">
         <v>222</v>
       </c>
-      <c r="F85" s="118"/>
-      <c r="G85" s="119">
-        <v>1</v>
-      </c>
-      <c r="H85" s="123"/>
-      <c r="I85" s="120" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="86" ht="15" customHeight="1">
-      <c r="B86" s="44" t="s">
+      <c r="F86" s="118"/>
+      <c r="G86" s="133">
+        <v>10</v>
+      </c>
+      <c r="H86" s="123"/>
+      <c r="I86" s="120" t="s">
         <v>304</v>
       </c>
-      <c r="C86" s="44"/>
-      <c r="D86" s="44"/>
-      <c r="E86" s="45"/>
-      <c r="F86" s="45"/>
-      <c r="G86" s="45"/>
-      <c r="H86" s="46"/>
-      <c r="I86" s="131" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="87" ht="15" customHeight="1">
-      <c r="B87" s="44"/>
-      <c r="C87" s="44"/>
-      <c r="D87" s="44"/>
-      <c r="E87" s="49" t="s">
-        <v>5</v>
-      </c>
-      <c r="F87" s="50" t="s">
-        <v>6</v>
-      </c>
-      <c r="G87" s="51" t="s">
-        <v>7</v>
-      </c>
-      <c r="H87" s="52"/>
-      <c r="I87" s="131"/>
+    </row>
+    <row r="87">
+      <c r="B87" s="126" t="s">
+        <v>305</v>
+      </c>
+      <c r="C87" s="126"/>
+      <c r="D87" s="126"/>
+      <c r="E87" s="117" t="s">
+        <v>222</v>
+      </c>
+      <c r="F87" s="118"/>
+      <c r="G87" s="133">
+        <v>10</v>
+      </c>
+      <c r="H87" s="123"/>
+      <c r="I87" s="120" t="s">
+        <v>304</v>
+      </c>
     </row>
     <row r="88">
-      <c r="B88" s="132" t="s">
-        <v>305</v>
-      </c>
-      <c r="C88" s="132"/>
-      <c r="D88" s="132"/>
+      <c r="B88" s="126" t="s">
+        <v>306</v>
+      </c>
+      <c r="C88" s="126"/>
+      <c r="D88" s="126"/>
       <c r="E88" s="117" t="s">
         <v>222</v>
       </c>
       <c r="F88" s="118"/>
       <c r="G88" s="133">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="H88" s="123"/>
       <c r="I88" s="120" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
     </row>
     <row r="89">
-      <c r="B89" s="126" t="s">
-        <v>307</v>
-      </c>
-      <c r="C89" s="126"/>
-      <c r="D89" s="126"/>
+      <c r="B89" s="122" t="s">
+        <v>308</v>
+      </c>
+      <c r="C89" s="122"/>
+      <c r="D89" s="122"/>
       <c r="E89" s="117" t="s">
         <v>222</v>
       </c>
       <c r="F89" s="118"/>
       <c r="G89" s="133">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="H89" s="123"/>
       <c r="I89" s="120" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
     </row>
     <row r="90">
-      <c r="B90" s="126" t="s">
-        <v>308</v>
-      </c>
-      <c r="C90" s="126"/>
-      <c r="D90" s="126"/>
+      <c r="B90" s="122" t="s">
+        <v>309</v>
+      </c>
+      <c r="C90" s="122"/>
+      <c r="D90" s="122"/>
       <c r="E90" s="117" t="s">
         <v>222</v>
       </c>
       <c r="F90" s="118"/>
       <c r="G90" s="133">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H90" s="123"/>
       <c r="I90" s="120" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="91">
@@ -9042,11 +9026,11 @@
       </c>
       <c r="F91" s="118"/>
       <c r="G91" s="133">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H91" s="123"/>
       <c r="I91" s="120" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="92">
@@ -9060,11 +9044,11 @@
       </c>
       <c r="F92" s="118"/>
       <c r="G92" s="133">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H92" s="123"/>
       <c r="I92" s="120" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="93">
@@ -9078,11 +9062,11 @@
       </c>
       <c r="F93" s="118"/>
       <c r="G93" s="133">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H93" s="123"/>
       <c r="I93" s="120" t="s">
-        <v>309</v>
+        <v>304</v>
       </c>
     </row>
     <row r="94">
@@ -9096,11 +9080,11 @@
       </c>
       <c r="F94" s="118"/>
       <c r="G94" s="133">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H94" s="123"/>
       <c r="I94" s="120" t="s">
-        <v>309</v>
+        <v>304</v>
       </c>
     </row>
     <row r="95">
@@ -9114,11 +9098,11 @@
       </c>
       <c r="F95" s="118"/>
       <c r="G95" s="133">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H95" s="123"/>
       <c r="I95" s="120" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
     </row>
     <row r="96">
@@ -9132,11 +9116,11 @@
       </c>
       <c r="F96" s="118"/>
       <c r="G96" s="133">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H96" s="123"/>
       <c r="I96" s="120" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
     </row>
     <row r="97">
@@ -9150,103 +9134,103 @@
       </c>
       <c r="F97" s="118"/>
       <c r="G97" s="133">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H97" s="123"/>
       <c r="I97" s="120" t="s">
-        <v>309</v>
+        <v>304</v>
       </c>
     </row>
     <row r="98">
-      <c r="B98" s="122" t="s">
+      <c r="B98" s="126" t="s">
         <v>317</v>
       </c>
-      <c r="C98" s="122"/>
-      <c r="D98" s="122"/>
+      <c r="C98" s="126"/>
+      <c r="D98" s="126"/>
       <c r="E98" s="117" t="s">
         <v>222</v>
       </c>
       <c r="F98" s="118"/>
       <c r="G98" s="133">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="H98" s="123"/>
       <c r="I98" s="120" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="99">
-      <c r="B99" s="122" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="99" ht="15" customHeight="1">
+      <c r="B99" s="44" t="s">
         <v>318</v>
       </c>
-      <c r="C99" s="122"/>
-      <c r="D99" s="122"/>
-      <c r="E99" s="117" t="s">
+      <c r="C99" s="44"/>
+      <c r="D99" s="44"/>
+      <c r="E99" s="45"/>
+      <c r="F99" s="45"/>
+      <c r="G99" s="45"/>
+      <c r="H99" s="46"/>
+      <c r="I99" s="131" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="100" ht="15" customHeight="1">
+      <c r="B100" s="44"/>
+      <c r="C100" s="44"/>
+      <c r="D100" s="44"/>
+      <c r="E100" s="49" t="s">
+        <v>5</v>
+      </c>
+      <c r="F100" s="50" t="s">
+        <v>6</v>
+      </c>
+      <c r="G100" s="51" t="s">
+        <v>7</v>
+      </c>
+      <c r="H100" s="52"/>
+      <c r="I100" s="131"/>
+    </row>
+    <row r="101">
+      <c r="B101" s="132" t="s">
+        <v>319</v>
+      </c>
+      <c r="C101" s="132"/>
+      <c r="D101" s="132"/>
+      <c r="E101" s="117" t="s">
         <v>222</v>
       </c>
-      <c r="F99" s="118"/>
-      <c r="G99" s="133">
-        <v>8</v>
-      </c>
-      <c r="H99" s="123"/>
-      <c r="I99" s="120" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="100">
-      <c r="B100" s="126" t="s">
-        <v>319</v>
-      </c>
-      <c r="C100" s="126"/>
-      <c r="D100" s="126"/>
-      <c r="E100" s="117" t="s">
+      <c r="F101" s="118"/>
+      <c r="G101" s="133">
+        <v>2</v>
+      </c>
+      <c r="H101" s="123"/>
+      <c r="I101" s="120" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="B102" s="126" t="s">
+        <v>320</v>
+      </c>
+      <c r="C102" s="126"/>
+      <c r="D102" s="126"/>
+      <c r="E102" s="117" t="s">
         <v>222</v>
       </c>
-      <c r="F100" s="118"/>
-      <c r="G100" s="133">
+      <c r="F102" s="118"/>
+      <c r="G102" s="133">
         <v>2</v>
       </c>
-      <c r="H100" s="123"/>
-      <c r="I100" s="120" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="101" ht="15" customHeight="1">
-      <c r="B101" s="44" t="s">
-        <v>320</v>
-      </c>
-      <c r="C101" s="44"/>
-      <c r="D101" s="44"/>
-      <c r="E101" s="45"/>
-      <c r="F101" s="45"/>
-      <c r="G101" s="45"/>
-      <c r="H101" s="46"/>
-      <c r="I101" s="131" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="102" ht="15" customHeight="1">
-      <c r="B102" s="44"/>
-      <c r="C102" s="44"/>
-      <c r="D102" s="44"/>
-      <c r="E102" s="49" t="s">
-        <v>5</v>
-      </c>
-      <c r="F102" s="50" t="s">
-        <v>6</v>
-      </c>
-      <c r="G102" s="51" t="s">
-        <v>7</v>
-      </c>
-      <c r="H102" s="52"/>
-      <c r="I102" s="131"/>
+      <c r="H102" s="123"/>
+      <c r="I102" s="120" t="s">
+        <v>252</v>
+      </c>
     </row>
     <row r="103">
-      <c r="B103" s="132" t="s">
+      <c r="B103" s="126" t="s">
         <v>321</v>
       </c>
-      <c r="C103" s="132"/>
-      <c r="D103" s="132"/>
+      <c r="C103" s="134"/>
+      <c r="D103" s="134"/>
       <c r="E103" s="117" t="s">
         <v>222</v>
       </c>
@@ -9263,8 +9247,8 @@
       <c r="B104" s="126" t="s">
         <v>322</v>
       </c>
-      <c r="C104" s="126"/>
-      <c r="D104" s="126"/>
+      <c r="C104" s="134"/>
+      <c r="D104" s="134"/>
       <c r="E104" s="117" t="s">
         <v>222</v>
       </c>
@@ -9342,11 +9326,11 @@
       </c>
       <c r="F108" s="118"/>
       <c r="G108" s="133">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H108" s="123"/>
       <c r="I108" s="120" t="s">
-        <v>252</v>
+        <v>304</v>
       </c>
     </row>
     <row r="109">
@@ -9360,11 +9344,11 @@
       </c>
       <c r="F109" s="118"/>
       <c r="G109" s="133">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H109" s="123"/>
       <c r="I109" s="120" t="s">
-        <v>252</v>
+        <v>304</v>
       </c>
     </row>
     <row r="110">
@@ -9382,81 +9366,81 @@
       </c>
       <c r="H110" s="123"/>
       <c r="I110" s="120" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="111">
-      <c r="B111" s="126" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="111" ht="14.25" customHeight="1">
+      <c r="B111" s="44" t="s">
         <v>329</v>
       </c>
-      <c r="C111" s="134"/>
-      <c r="D111" s="134"/>
-      <c r="E111" s="117" t="s">
+      <c r="C111" s="44"/>
+      <c r="D111" s="44"/>
+      <c r="E111" s="45"/>
+      <c r="F111" s="45"/>
+      <c r="G111" s="45"/>
+      <c r="H111" s="46"/>
+      <c r="I111" s="131" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="112" ht="15" customHeight="1">
+      <c r="B112" s="44"/>
+      <c r="C112" s="44"/>
+      <c r="D112" s="44"/>
+      <c r="E112" s="49" t="s">
+        <v>5</v>
+      </c>
+      <c r="F112" s="50" t="s">
+        <v>6</v>
+      </c>
+      <c r="G112" s="51" t="s">
+        <v>7</v>
+      </c>
+      <c r="H112" s="52"/>
+      <c r="I112" s="131"/>
+    </row>
+    <row r="113">
+      <c r="B113" s="132" t="s">
+        <v>330</v>
+      </c>
+      <c r="C113" s="132"/>
+      <c r="D113" s="132"/>
+      <c r="E113" s="117" t="s">
         <v>222</v>
       </c>
-      <c r="F111" s="118"/>
-      <c r="G111" s="133">
-        <v>3</v>
-      </c>
-      <c r="H111" s="123"/>
-      <c r="I111" s="120" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="112">
-      <c r="B112" s="126" t="s">
-        <v>330</v>
-      </c>
-      <c r="C112" s="134"/>
-      <c r="D112" s="134"/>
-      <c r="E112" s="117" t="s">
+      <c r="F113" s="118"/>
+      <c r="G113" s="133">
+        <v>1</v>
+      </c>
+      <c r="H113" s="123"/>
+      <c r="I113" s="120" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="B114" s="126" t="s">
+        <v>331</v>
+      </c>
+      <c r="C114" s="126"/>
+      <c r="D114" s="126"/>
+      <c r="E114" s="117" t="s">
         <v>222</v>
       </c>
-      <c r="F112" s="118"/>
-      <c r="G112" s="133">
-        <v>3</v>
-      </c>
-      <c r="H112" s="123"/>
-      <c r="I112" s="120" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="113" ht="14.25" customHeight="1">
-      <c r="B113" s="44" t="s">
-        <v>331</v>
-      </c>
-      <c r="C113" s="44"/>
-      <c r="D113" s="44"/>
-      <c r="E113" s="45"/>
-      <c r="F113" s="45"/>
-      <c r="G113" s="45"/>
-      <c r="H113" s="46"/>
-      <c r="I113" s="131" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="114" ht="15" customHeight="1">
-      <c r="B114" s="44"/>
-      <c r="C114" s="44"/>
-      <c r="D114" s="44"/>
-      <c r="E114" s="49" t="s">
-        <v>5</v>
-      </c>
-      <c r="F114" s="50" t="s">
-        <v>6</v>
-      </c>
-      <c r="G114" s="51" t="s">
-        <v>7</v>
-      </c>
-      <c r="H114" s="52"/>
-      <c r="I114" s="131"/>
+      <c r="F114" s="118"/>
+      <c r="G114" s="133">
+        <v>1</v>
+      </c>
+      <c r="H114" s="123"/>
+      <c r="I114" s="120" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="115">
-      <c r="B115" s="132" t="s">
+      <c r="B115" s="126" t="s">
         <v>332</v>
       </c>
-      <c r="C115" s="132"/>
-      <c r="D115" s="132"/>
+      <c r="C115" s="126"/>
+      <c r="D115" s="126"/>
       <c r="E115" s="117" t="s">
         <v>222</v>
       </c>
@@ -9556,7 +9540,7 @@
       </c>
       <c r="H120" s="123"/>
       <c r="I120" s="120" t="s">
-        <v>224</v>
+        <v>250</v>
       </c>
     </row>
     <row r="121">
@@ -9574,7 +9558,7 @@
       </c>
       <c r="H121" s="123"/>
       <c r="I121" s="120" t="s">
-        <v>224</v>
+        <v>250</v>
       </c>
     </row>
     <row r="122">
@@ -9602,15 +9586,15 @@
       <c r="C123" s="126"/>
       <c r="D123" s="126"/>
       <c r="E123" s="117" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="F123" s="118"/>
       <c r="G123" s="133">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H123" s="123"/>
       <c r="I123" s="120" t="s">
-        <v>250</v>
+        <v>224</v>
       </c>
     </row>
     <row r="124">
@@ -9638,11 +9622,11 @@
       <c r="C125" s="126"/>
       <c r="D125" s="126"/>
       <c r="E125" s="117" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="F125" s="118"/>
       <c r="G125" s="133">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H125" s="123"/>
       <c r="I125" s="120" t="s">
@@ -9656,97 +9640,91 @@
       <c r="C126" s="126"/>
       <c r="D126" s="126"/>
       <c r="E126" s="117" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="F126" s="118"/>
       <c r="G126" s="133">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H126" s="123"/>
       <c r="I126" s="120" t="s">
         <v>250</v>
       </c>
     </row>
-    <row r="127">
-      <c r="B127" s="126" t="s">
+    <row r="127" ht="14.25" customHeight="1">
+      <c r="B127" s="44" t="s">
         <v>344</v>
       </c>
-      <c r="C127" s="126"/>
-      <c r="D127" s="126"/>
-      <c r="E127" s="117" t="s">
-        <v>227</v>
-      </c>
-      <c r="F127" s="118"/>
-      <c r="G127" s="133">
-        <v>2</v>
-      </c>
-      <c r="H127" s="123"/>
-      <c r="I127" s="120" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="128">
-      <c r="B128" s="126" t="s">
-        <v>345</v>
-      </c>
-      <c r="C128" s="126"/>
-      <c r="D128" s="126"/>
-      <c r="E128" s="117" t="s">
-        <v>222</v>
-      </c>
-      <c r="F128" s="118"/>
-      <c r="G128" s="133">
-        <v>1</v>
-      </c>
-      <c r="H128" s="123"/>
-      <c r="I128" s="120" t="s">
-        <v>250</v>
-      </c>
+      <c r="C127" s="44"/>
+      <c r="D127" s="44"/>
+      <c r="E127" s="45"/>
+      <c r="F127" s="45"/>
+      <c r="G127" s="45"/>
+      <c r="H127" s="46"/>
+      <c r="I127" s="131" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="128" ht="15" customHeight="1">
+      <c r="B128" s="44"/>
+      <c r="C128" s="44"/>
+      <c r="D128" s="44"/>
+      <c r="E128" s="49" t="s">
+        <v>5</v>
+      </c>
+      <c r="F128" s="50" t="s">
+        <v>6</v>
+      </c>
+      <c r="G128" s="51" t="s">
+        <v>7</v>
+      </c>
+      <c r="H128" s="52"/>
+      <c r="I128" s="131"/>
     </row>
     <row r="129">
-      <c r="B129" s="126" t="s">
-        <v>346</v>
-      </c>
-      <c r="C129" s="126"/>
-      <c r="D129" s="126"/>
+      <c r="B129" s="135" t="s">
+        <v>202</v>
+      </c>
+      <c r="C129" s="135"/>
+      <c r="D129" s="135"/>
       <c r="E129" s="117" t="s">
         <v>222</v>
       </c>
       <c r="F129" s="118"/>
       <c r="G129" s="133">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H129" s="123"/>
       <c r="I129" s="120" t="s">
-        <v>224</v>
+        <v>345</v>
       </c>
     </row>
     <row r="130">
-      <c r="B130" s="126" t="s">
-        <v>347</v>
-      </c>
-      <c r="C130" s="126"/>
-      <c r="D130" s="126"/>
+      <c r="B130" s="122" t="s">
+        <v>210</v>
+      </c>
+      <c r="C130" s="122"/>
+      <c r="D130" s="122"/>
       <c r="E130" s="117" t="s">
         <v>222</v>
       </c>
       <c r="F130" s="118"/>
       <c r="G130" s="133">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H130" s="123"/>
       <c r="I130" s="120" t="s">
-        <v>250</v>
+        <v>346</v>
       </c>
     </row>
     <row r="131">
-      <c r="B131" s="126" t="s">
-        <v>348</v>
-      </c>
-      <c r="C131" s="126"/>
-      <c r="D131" s="126"/>
+      <c r="B131" s="136" t="s">
+        <v>209</v>
+      </c>
+      <c r="C131" s="137"/>
+      <c r="D131" s="138"/>
       <c r="E131" s="117" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="F131" s="118"/>
       <c r="G131" s="133">
@@ -9754,45 +9732,51 @@
       </c>
       <c r="H131" s="123"/>
       <c r="I131" s="120" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="132" ht="14.25" customHeight="1">
-      <c r="B132" s="44" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="B132" s="120" t="s">
+        <v>348</v>
+      </c>
+      <c r="C132" s="120"/>
+      <c r="D132" s="120"/>
+      <c r="E132" s="117" t="s">
+        <v>222</v>
+      </c>
+      <c r="F132" s="118"/>
+      <c r="G132" s="133">
+        <v>4</v>
+      </c>
+      <c r="H132" s="123"/>
+      <c r="I132" s="120" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="B133" s="136" t="s">
         <v>349</v>
       </c>
-      <c r="C132" s="44"/>
-      <c r="D132" s="44"/>
-      <c r="E132" s="45"/>
-      <c r="F132" s="45"/>
-      <c r="G132" s="45"/>
-      <c r="H132" s="46"/>
-      <c r="I132" s="131" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="133" ht="15" customHeight="1">
-      <c r="B133" s="44"/>
-      <c r="C133" s="44"/>
-      <c r="D133" s="44"/>
-      <c r="E133" s="49" t="s">
-        <v>5</v>
-      </c>
-      <c r="F133" s="50" t="s">
-        <v>6</v>
-      </c>
-      <c r="G133" s="51" t="s">
-        <v>7</v>
-      </c>
-      <c r="H133" s="52"/>
-      <c r="I133" s="131"/>
+      <c r="C133" s="137"/>
+      <c r="D133" s="138"/>
+      <c r="E133" s="117" t="s">
+        <v>222</v>
+      </c>
+      <c r="F133" s="118"/>
+      <c r="G133" s="133">
+        <v>4</v>
+      </c>
+      <c r="H133" s="123"/>
+      <c r="I133" s="120" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="134">
-      <c r="B134" s="135" t="s">
-        <v>202</v>
-      </c>
-      <c r="C134" s="135"/>
-      <c r="D134" s="135"/>
+      <c r="B134" s="136" t="s">
+        <v>350</v>
+      </c>
+      <c r="C134" s="137"/>
+      <c r="D134" s="138"/>
       <c r="E134" s="117" t="s">
         <v>222</v>
       </c>
@@ -9802,15 +9786,15 @@
       </c>
       <c r="H134" s="123"/>
       <c r="I134" s="120" t="s">
-        <v>350</v>
+        <v>13</v>
       </c>
     </row>
     <row r="135">
-      <c r="B135" s="122" t="s">
-        <v>210</v>
-      </c>
-      <c r="C135" s="122"/>
-      <c r="D135" s="122"/>
+      <c r="B135" s="136" t="s">
+        <v>351</v>
+      </c>
+      <c r="C135" s="137"/>
+      <c r="D135" s="138"/>
       <c r="E135" s="117" t="s">
         <v>222</v>
       </c>
@@ -9820,12 +9804,12 @@
       </c>
       <c r="H135" s="123"/>
       <c r="I135" s="120" t="s">
-        <v>351</v>
+        <v>13</v>
       </c>
     </row>
     <row r="136">
       <c r="B136" s="136" t="s">
-        <v>209</v>
+        <v>352</v>
       </c>
       <c r="C136" s="137"/>
       <c r="D136" s="138"/>
@@ -9834,19 +9818,19 @@
       </c>
       <c r="F136" s="118"/>
       <c r="G136" s="133">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H136" s="123"/>
       <c r="I136" s="120" t="s">
-        <v>352</v>
+        <v>13</v>
       </c>
     </row>
     <row r="137">
-      <c r="B137" s="120" t="s">
+      <c r="B137" s="136" t="s">
         <v>353</v>
       </c>
-      <c r="C137" s="120"/>
-      <c r="D137" s="120"/>
+      <c r="C137" s="137"/>
+      <c r="D137" s="138"/>
       <c r="E137" s="117" t="s">
         <v>222</v>
       </c>
@@ -9932,17 +9916,17 @@
       </c>
     </row>
     <row r="142">
-      <c r="B142" s="136" t="s">
+      <c r="B142" s="120" t="s">
         <v>358</v>
       </c>
-      <c r="C142" s="137"/>
-      <c r="D142" s="138"/>
+      <c r="C142" s="120"/>
+      <c r="D142" s="120"/>
       <c r="E142" s="117" t="s">
         <v>222</v>
       </c>
       <c r="F142" s="118"/>
       <c r="G142" s="133">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H142" s="123"/>
       <c r="I142" s="120" t="s">
@@ -9950,17 +9934,17 @@
       </c>
     </row>
     <row r="143">
-      <c r="B143" s="136" t="s">
+      <c r="B143" s="120" t="s">
         <v>359</v>
       </c>
-      <c r="C143" s="137"/>
-      <c r="D143" s="138"/>
+      <c r="C143" s="120"/>
+      <c r="D143" s="120"/>
       <c r="E143" s="117" t="s">
         <v>222</v>
       </c>
       <c r="F143" s="118"/>
       <c r="G143" s="133">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H143" s="123"/>
       <c r="I143" s="120" t="s">
@@ -9968,17 +9952,17 @@
       </c>
     </row>
     <row r="144">
-      <c r="B144" s="136" t="s">
+      <c r="B144" s="120" t="s">
         <v>360</v>
       </c>
-      <c r="C144" s="137"/>
-      <c r="D144" s="138"/>
+      <c r="C144" s="120"/>
+      <c r="D144" s="120"/>
       <c r="E144" s="117" t="s">
         <v>222</v>
       </c>
       <c r="F144" s="118"/>
       <c r="G144" s="133">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H144" s="123"/>
       <c r="I144" s="120" t="s">
@@ -9986,17 +9970,17 @@
       </c>
     </row>
     <row r="145">
-      <c r="B145" s="136" t="s">
+      <c r="B145" s="120" t="s">
         <v>361</v>
       </c>
-      <c r="C145" s="137"/>
-      <c r="D145" s="138"/>
+      <c r="C145" s="120"/>
+      <c r="D145" s="120"/>
       <c r="E145" s="117" t="s">
         <v>222</v>
       </c>
       <c r="F145" s="118"/>
       <c r="G145" s="133">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H145" s="123"/>
       <c r="I145" s="120" t="s">
@@ -10004,17 +9988,17 @@
       </c>
     </row>
     <row r="146">
-      <c r="B146" s="136" t="s">
+      <c r="B146" s="120" t="s">
         <v>362</v>
       </c>
-      <c r="C146" s="137"/>
-      <c r="D146" s="138"/>
+      <c r="C146" s="120"/>
+      <c r="D146" s="120"/>
       <c r="E146" s="117" t="s">
-        <v>222</v>
+        <v>363</v>
       </c>
       <c r="F146" s="118"/>
       <c r="G146" s="133">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H146" s="123"/>
       <c r="I146" s="120" t="s">
@@ -10022,17 +10006,17 @@
       </c>
     </row>
     <row r="147">
-      <c r="B147" s="120" t="s">
+      <c r="B147" s="136" t="s">
+        <v>364</v>
+      </c>
+      <c r="C147" s="137"/>
+      <c r="D147" s="138"/>
+      <c r="E147" s="117" t="s">
         <v>363</v>
-      </c>
-      <c r="C147" s="120"/>
-      <c r="D147" s="120"/>
-      <c r="E147" s="117" t="s">
-        <v>222</v>
       </c>
       <c r="F147" s="118"/>
       <c r="G147" s="133">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H147" s="123"/>
       <c r="I147" s="120" t="s">
@@ -10040,17 +10024,17 @@
       </c>
     </row>
     <row r="148">
-      <c r="B148" s="120" t="s">
-        <v>364</v>
-      </c>
-      <c r="C148" s="120"/>
-      <c r="D148" s="120"/>
+      <c r="B148" s="136" t="s">
+        <v>365</v>
+      </c>
+      <c r="C148" s="137"/>
+      <c r="D148" s="138"/>
       <c r="E148" s="117" t="s">
-        <v>222</v>
+        <v>363</v>
       </c>
       <c r="F148" s="118"/>
       <c r="G148" s="133">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H148" s="123"/>
       <c r="I148" s="120" t="s">
@@ -10058,13 +10042,13 @@
       </c>
     </row>
     <row r="149">
-      <c r="B149" s="120" t="s">
-        <v>365</v>
-      </c>
-      <c r="C149" s="120"/>
-      <c r="D149" s="120"/>
+      <c r="B149" s="136" t="s">
+        <v>366</v>
+      </c>
+      <c r="C149" s="137"/>
+      <c r="D149" s="138"/>
       <c r="E149" s="117" t="s">
-        <v>222</v>
+        <v>363</v>
       </c>
       <c r="F149" s="118"/>
       <c r="G149" s="133">
@@ -10076,31 +10060,31 @@
       </c>
     </row>
     <row r="150">
-      <c r="B150" s="120" t="s">
-        <v>366</v>
-      </c>
-      <c r="C150" s="120"/>
-      <c r="D150" s="120"/>
+      <c r="B150" s="136" t="s">
+        <v>367</v>
+      </c>
+      <c r="C150" s="137"/>
+      <c r="D150" s="138"/>
       <c r="E150" s="117" t="s">
         <v>222</v>
       </c>
       <c r="F150" s="118"/>
       <c r="G150" s="133">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H150" s="123"/>
       <c r="I150" s="120" t="s">
-        <v>13</v>
+        <v>347</v>
       </c>
     </row>
     <row r="151">
-      <c r="B151" s="120" t="s">
-        <v>367</v>
-      </c>
-      <c r="C151" s="120"/>
-      <c r="D151" s="120"/>
+      <c r="B151" s="136" t="s">
+        <v>368</v>
+      </c>
+      <c r="C151" s="137"/>
+      <c r="D151" s="138"/>
       <c r="E151" s="117" t="s">
-        <v>368</v>
+        <v>222</v>
       </c>
       <c r="F151" s="118"/>
       <c r="G151" s="133">
@@ -10108,17 +10092,17 @@
       </c>
       <c r="H151" s="123"/>
       <c r="I151" s="120" t="s">
-        <v>13</v>
+        <v>347</v>
       </c>
     </row>
     <row r="152">
-      <c r="B152" s="136" t="s">
+      <c r="B152" s="126" t="s">
         <v>369</v>
       </c>
-      <c r="C152" s="137"/>
-      <c r="D152" s="138"/>
+      <c r="C152" s="126"/>
+      <c r="D152" s="126"/>
       <c r="E152" s="117" t="s">
-        <v>368</v>
+        <v>222</v>
       </c>
       <c r="F152" s="118"/>
       <c r="G152" s="133">
@@ -10126,17 +10110,17 @@
       </c>
       <c r="H152" s="123"/>
       <c r="I152" s="120" t="s">
-        <v>13</v>
+        <v>347</v>
       </c>
     </row>
     <row r="153">
-      <c r="B153" s="136" t="s">
+      <c r="B153" s="126" t="s">
         <v>370</v>
       </c>
-      <c r="C153" s="137"/>
-      <c r="D153" s="138"/>
+      <c r="C153" s="126"/>
+      <c r="D153" s="126"/>
       <c r="E153" s="117" t="s">
-        <v>368</v>
+        <v>222</v>
       </c>
       <c r="F153" s="118"/>
       <c r="G153" s="133">
@@ -10144,21 +10128,21 @@
       </c>
       <c r="H153" s="123"/>
       <c r="I153" s="120" t="s">
-        <v>13</v>
+        <v>347</v>
       </c>
     </row>
     <row r="154">
-      <c r="B154" s="136" t="s">
+      <c r="B154" s="126" t="s">
         <v>371</v>
       </c>
-      <c r="C154" s="137"/>
-      <c r="D154" s="138"/>
+      <c r="C154" s="126"/>
+      <c r="D154" s="126"/>
       <c r="E154" s="117" t="s">
-        <v>368</v>
+        <v>222</v>
       </c>
       <c r="F154" s="118"/>
       <c r="G154" s="133">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H154" s="123"/>
       <c r="I154" s="120" t="s">
@@ -10166,13 +10150,13 @@
       </c>
     </row>
     <row r="155">
-      <c r="B155" s="136" t="s">
+      <c r="B155" s="126" t="s">
         <v>372</v>
       </c>
-      <c r="C155" s="137"/>
-      <c r="D155" s="138"/>
+      <c r="C155" s="126"/>
+      <c r="D155" s="126"/>
       <c r="E155" s="117" t="s">
-        <v>368</v>
+        <v>222</v>
       </c>
       <c r="F155" s="118"/>
       <c r="G155" s="133">
@@ -10184,11 +10168,11 @@
       </c>
     </row>
     <row r="156">
-      <c r="B156" s="136" t="s">
+      <c r="B156" s="126" t="s">
         <v>373</v>
       </c>
-      <c r="C156" s="137"/>
-      <c r="D156" s="138"/>
+      <c r="C156" s="126"/>
+      <c r="D156" s="126"/>
       <c r="E156" s="117" t="s">
         <v>222</v>
       </c>
@@ -10198,15 +10182,15 @@
       </c>
       <c r="H156" s="123"/>
       <c r="I156" s="120" t="s">
-        <v>352</v>
+        <v>13</v>
       </c>
     </row>
     <row r="157">
-      <c r="B157" s="136" t="s">
+      <c r="B157" s="126" t="s">
         <v>374</v>
       </c>
-      <c r="C157" s="137"/>
-      <c r="D157" s="138"/>
+      <c r="C157" s="126"/>
+      <c r="D157" s="126"/>
       <c r="E157" s="117" t="s">
         <v>222</v>
       </c>
@@ -10216,7 +10200,7 @@
       </c>
       <c r="H157" s="123"/>
       <c r="I157" s="120" t="s">
-        <v>352</v>
+        <v>252</v>
       </c>
     </row>
     <row r="158">
@@ -10234,7 +10218,7 @@
       </c>
       <c r="H158" s="123"/>
       <c r="I158" s="120" t="s">
-        <v>352</v>
+        <v>252</v>
       </c>
     </row>
     <row r="159">
@@ -10252,7 +10236,7 @@
       </c>
       <c r="H159" s="123"/>
       <c r="I159" s="120" t="s">
-        <v>352</v>
+        <v>252</v>
       </c>
     </row>
     <row r="160">
@@ -10266,11 +10250,11 @@
       </c>
       <c r="F160" s="118"/>
       <c r="G160" s="133">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H160" s="123"/>
       <c r="I160" s="120" t="s">
-        <v>13</v>
+        <v>252</v>
       </c>
     </row>
     <row r="161">
@@ -10288,7 +10272,7 @@
       </c>
       <c r="H161" s="123"/>
       <c r="I161" s="120" t="s">
-        <v>13</v>
+        <v>252</v>
       </c>
     </row>
     <row r="162">
@@ -10306,7 +10290,7 @@
       </c>
       <c r="H162" s="123"/>
       <c r="I162" s="120" t="s">
-        <v>13</v>
+        <v>252</v>
       </c>
     </row>
     <row r="163">
@@ -10328,172 +10312,106 @@
       </c>
     </row>
     <row r="164">
-      <c r="B164" s="126" t="s">
-        <v>381</v>
-      </c>
-      <c r="C164" s="126"/>
-      <c r="D164" s="126"/>
-      <c r="E164" s="117" t="s">
-        <v>222</v>
-      </c>
-      <c r="F164" s="118"/>
-      <c r="G164" s="133">
-        <v>2</v>
-      </c>
-      <c r="H164" s="123"/>
-      <c r="I164" s="120" t="s">
-        <v>252</v>
-      </c>
+      <c r="E164" s="2"/>
+      <c r="F164" s="4"/>
+      <c r="G164" s="109"/>
+      <c r="H164" s="6"/>
+      <c r="I164" s="110"/>
     </row>
     <row r="165">
-      <c r="B165" s="126" t="s">
-        <v>382</v>
-      </c>
-      <c r="C165" s="126"/>
-      <c r="D165" s="126"/>
-      <c r="E165" s="117" t="s">
-        <v>222</v>
-      </c>
-      <c r="F165" s="118"/>
-      <c r="G165" s="133">
-        <v>2</v>
-      </c>
-      <c r="H165" s="123"/>
-      <c r="I165" s="120" t="s">
-        <v>252</v>
-      </c>
+      <c r="D165" s="103"/>
+      <c r="E165" s="139"/>
+      <c r="F165" s="140"/>
+      <c r="G165" s="141"/>
+      <c r="H165" s="140"/>
+      <c r="I165" s="140"/>
     </row>
     <row r="166">
-      <c r="B166" s="126" t="s">
-        <v>383</v>
-      </c>
-      <c r="C166" s="126"/>
-      <c r="D166" s="126"/>
-      <c r="E166" s="117" t="s">
-        <v>222</v>
-      </c>
-      <c r="F166" s="118"/>
-      <c r="G166" s="133">
-        <v>2</v>
-      </c>
-      <c r="H166" s="123"/>
-      <c r="I166" s="120" t="s">
-        <v>252</v>
-      </c>
+      <c r="D166" s="103"/>
+      <c r="E166" s="103"/>
+      <c r="F166" s="103"/>
+      <c r="H166" s="142"/>
     </row>
     <row r="167">
-      <c r="B167" s="126" t="s">
-        <v>384</v>
-      </c>
-      <c r="C167" s="126"/>
-      <c r="D167" s="126"/>
-      <c r="E167" s="117" t="s">
-        <v>222</v>
-      </c>
-      <c r="F167" s="118"/>
-      <c r="G167" s="133">
-        <v>2</v>
-      </c>
-      <c r="H167" s="123"/>
-      <c r="I167" s="120" t="s">
-        <v>252</v>
-      </c>
+      <c r="D167" s="103"/>
+      <c r="E167" s="103"/>
+      <c r="F167" s="103"/>
+      <c r="H167" s="142"/>
     </row>
     <row r="168">
-      <c r="B168" s="126" t="s">
-        <v>385</v>
-      </c>
-      <c r="C168" s="126"/>
-      <c r="D168" s="126"/>
-      <c r="E168" s="117" t="s">
-        <v>222</v>
-      </c>
-      <c r="F168" s="118"/>
-      <c r="G168" s="133">
-        <v>2</v>
-      </c>
-      <c r="H168" s="123"/>
-      <c r="I168" s="120" t="s">
-        <v>252</v>
-      </c>
+      <c r="D168" s="103"/>
+      <c r="E168" s="103"/>
+      <c r="F168" s="103"/>
+      <c r="H168" s="142"/>
     </row>
     <row r="169">
-      <c r="B169" s="126" t="s">
-        <v>386</v>
-      </c>
-      <c r="C169" s="126"/>
-      <c r="D169" s="126"/>
-      <c r="E169" s="117" t="s">
-        <v>222</v>
-      </c>
-      <c r="F169" s="118"/>
-      <c r="G169" s="133">
-        <v>2</v>
-      </c>
-      <c r="H169" s="123"/>
-      <c r="I169" s="120" t="s">
-        <v>252</v>
-      </c>
+      <c r="D169" s="103"/>
+      <c r="E169" s="103"/>
+      <c r="F169" s="103"/>
+      <c r="H169" s="142"/>
     </row>
     <row r="170">
-      <c r="E170" s="2"/>
-      <c r="F170" s="4"/>
-      <c r="G170" s="109"/>
-      <c r="H170" s="6"/>
-      <c r="I170" s="110"/>
+      <c r="D170" s="103"/>
+      <c r="E170" s="139"/>
+      <c r="F170" s="140"/>
+      <c r="G170" s="143"/>
+      <c r="H170" s="141"/>
     </row>
     <row r="171">
       <c r="D171" s="103"/>
-      <c r="E171" s="139"/>
-      <c r="F171" s="140"/>
-      <c r="G171" s="141"/>
-      <c r="H171" s="140"/>
-      <c r="I171" s="140"/>
+      <c r="H171" s="142"/>
     </row>
     <row r="172">
+      <c r="B172" s="1" t="s">
+        <v>2</v>
+      </c>
       <c r="D172" s="103"/>
-      <c r="E172" s="103"/>
-      <c r="F172" s="103"/>
-      <c r="H172" s="142"/>
+      <c r="E172" s="139"/>
+      <c r="F172" s="140"/>
+      <c r="G172" s="143"/>
+      <c r="H172" s="141"/>
     </row>
     <row r="173">
-      <c r="D173" s="103"/>
-      <c r="E173" s="103"/>
-      <c r="F173" s="103"/>
-      <c r="H173" s="142"/>
+      <c r="E173" s="2"/>
+      <c r="F173" s="4"/>
+      <c r="G173" s="109"/>
+      <c r="H173" s="6"/>
+      <c r="I173" s="110"/>
     </row>
     <row r="174">
-      <c r="D174" s="103"/>
-      <c r="E174" s="103"/>
-      <c r="F174" s="103"/>
-      <c r="H174" s="142"/>
+      <c r="E174" s="2"/>
+      <c r="F174" s="4"/>
+      <c r="G174" s="109"/>
+      <c r="H174" s="6"/>
+      <c r="I174" s="110"/>
     </row>
     <row r="175">
-      <c r="D175" s="103"/>
-      <c r="E175" s="103"/>
-      <c r="F175" s="103"/>
-      <c r="H175" s="142"/>
+      <c r="E175" s="2"/>
+      <c r="F175" s="4"/>
+      <c r="G175" s="109"/>
+      <c r="H175" s="6"/>
+      <c r="I175" s="110"/>
     </row>
     <row r="176">
-      <c r="D176" s="103"/>
-      <c r="E176" s="139"/>
-      <c r="F176" s="140"/>
-      <c r="G176" s="143"/>
-      <c r="H176" s="141"/>
+      <c r="E176" s="2"/>
+      <c r="F176" s="4"/>
+      <c r="G176" s="109"/>
+      <c r="H176" s="6"/>
+      <c r="I176" s="110"/>
     </row>
     <row r="177">
-      <c r="D177" s="103"/>
-      <c r="H177" s="142"/>
+      <c r="E177" s="2"/>
+      <c r="F177" s="4"/>
+      <c r="G177" s="109"/>
+      <c r="H177" s="6"/>
+      <c r="I177" s="110"/>
     </row>
     <row r="178">
-      <c r="B178" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D178" s="103"/>
-      <c r="E178" s="139"/>
-      <c r="F178" s="140"/>
-      <c r="G178" s="143"/>
-      <c r="H178" s="141"/>
+      <c r="E178" s="2"/>
+      <c r="F178" s="4"/>
+      <c r="G178" s="109"/>
+      <c r="H178" s="6"/>
+      <c r="I178" s="110"/>
     </row>
     <row r="179">
       <c r="E179" s="2"/>
@@ -10740,47 +10658,53 @@
       <c r="H213" s="6"/>
       <c r="I213" s="110"/>
     </row>
-    <row r="214">
+    <row r="214" s="1" customFormat="1">
       <c r="E214" s="2"/>
       <c r="F214" s="4"/>
       <c r="G214" s="109"/>
       <c r="H214" s="6"/>
       <c r="I214" s="110"/>
-    </row>
-    <row r="215">
+      <c r="W214" s="103"/>
+    </row>
+    <row r="215" s="1" customFormat="1">
       <c r="E215" s="2"/>
       <c r="F215" s="4"/>
       <c r="G215" s="109"/>
       <c r="H215" s="6"/>
       <c r="I215" s="110"/>
-    </row>
-    <row r="216">
+      <c r="W215" s="103"/>
+    </row>
+    <row r="216" s="1" customFormat="1">
       <c r="E216" s="2"/>
       <c r="F216" s="4"/>
       <c r="G216" s="109"/>
       <c r="H216" s="6"/>
       <c r="I216" s="110"/>
-    </row>
-    <row r="217">
+      <c r="W216" s="103"/>
+    </row>
+    <row r="217" s="1" customFormat="1">
       <c r="E217" s="2"/>
       <c r="F217" s="4"/>
       <c r="G217" s="109"/>
       <c r="H217" s="6"/>
       <c r="I217" s="110"/>
-    </row>
-    <row r="218">
+      <c r="W217" s="103"/>
+    </row>
+    <row r="218" s="1" customFormat="1">
       <c r="E218" s="2"/>
       <c r="F218" s="4"/>
       <c r="G218" s="109"/>
       <c r="H218" s="6"/>
       <c r="I218" s="110"/>
-    </row>
-    <row r="219">
+      <c r="W218" s="103"/>
+    </row>
+    <row r="219" s="1" customFormat="1">
       <c r="E219" s="2"/>
       <c r="F219" s="4"/>
       <c r="G219" s="109"/>
       <c r="H219" s="6"/>
       <c r="I219" s="110"/>
+      <c r="W219" s="103"/>
     </row>
     <row r="220" s="1" customFormat="1">
       <c r="E220" s="2"/>
@@ -11766,53 +11690,35 @@
       <c r="I342" s="110"/>
       <c r="W342" s="103"/>
     </row>
-    <row r="343" s="1" customFormat="1">
+    <row r="343">
       <c r="E343" s="2"/>
       <c r="F343" s="4"/>
       <c r="G343" s="109"/>
-      <c r="H343" s="6"/>
-      <c r="I343" s="110"/>
-      <c r="W343" s="103"/>
-    </row>
-    <row r="344" s="1" customFormat="1">
+    </row>
+    <row r="344">
       <c r="E344" s="2"/>
       <c r="F344" s="4"/>
       <c r="G344" s="109"/>
-      <c r="H344" s="6"/>
-      <c r="I344" s="110"/>
-      <c r="W344" s="103"/>
-    </row>
-    <row r="345" s="1" customFormat="1">
+    </row>
+    <row r="345">
       <c r="E345" s="2"/>
       <c r="F345" s="4"/>
       <c r="G345" s="109"/>
-      <c r="H345" s="6"/>
-      <c r="I345" s="110"/>
-      <c r="W345" s="103"/>
-    </row>
-    <row r="346" s="1" customFormat="1">
+    </row>
+    <row r="346">
       <c r="E346" s="2"/>
       <c r="F346" s="4"/>
       <c r="G346" s="109"/>
-      <c r="H346" s="6"/>
-      <c r="I346" s="110"/>
-      <c r="W346" s="103"/>
-    </row>
-    <row r="347" s="1" customFormat="1">
+    </row>
+    <row r="347">
       <c r="E347" s="2"/>
       <c r="F347" s="4"/>
       <c r="G347" s="109"/>
-      <c r="H347" s="6"/>
-      <c r="I347" s="110"/>
-      <c r="W347" s="103"/>
-    </row>
-    <row r="348" s="1" customFormat="1">
+    </row>
+    <row r="348">
       <c r="E348" s="2"/>
       <c r="F348" s="4"/>
       <c r="G348" s="109"/>
-      <c r="H348" s="6"/>
-      <c r="I348" s="110"/>
-      <c r="W348" s="103"/>
     </row>
     <row r="349">
       <c r="E349" s="2"/>
@@ -12874,38 +12780,8 @@
       <c r="F560" s="4"/>
       <c r="G560" s="109"/>
     </row>
-    <row r="561">
-      <c r="E561" s="2"/>
-      <c r="F561" s="4"/>
-      <c r="G561" s="109"/>
-    </row>
-    <row r="562">
-      <c r="E562" s="2"/>
-      <c r="F562" s="4"/>
-      <c r="G562" s="109"/>
-    </row>
-    <row r="563">
-      <c r="E563" s="2"/>
-      <c r="F563" s="4"/>
-      <c r="G563" s="109"/>
-    </row>
-    <row r="564">
-      <c r="E564" s="2"/>
-      <c r="F564" s="4"/>
-      <c r="G564" s="109"/>
-    </row>
-    <row r="565">
-      <c r="E565" s="2"/>
-      <c r="F565" s="4"/>
-      <c r="G565" s="109"/>
-    </row>
-    <row r="566">
-      <c r="E566" s="2"/>
-      <c r="F566" s="4"/>
-      <c r="G566" s="109"/>
-    </row>
   </sheetData>
-  <mergeCells count="66">
+  <mergeCells count="65">
     <mergeCell ref="B5:D6"/>
     <mergeCell ref="E5:G5"/>
     <mergeCell ref="I5:I6"/>
@@ -12927,55 +12803,54 @@
     <mergeCell ref="B24:D24"/>
     <mergeCell ref="B25:D25"/>
     <mergeCell ref="B32:D32"/>
-    <mergeCell ref="B85:D85"/>
-    <mergeCell ref="B86:D87"/>
-    <mergeCell ref="E86:G86"/>
-    <mergeCell ref="I86:I87"/>
+    <mergeCell ref="B83:D83"/>
+    <mergeCell ref="B84:D85"/>
+    <mergeCell ref="E84:G84"/>
+    <mergeCell ref="I84:I85"/>
+    <mergeCell ref="B86:D86"/>
+    <mergeCell ref="B87:D87"/>
     <mergeCell ref="B88:D88"/>
     <mergeCell ref="B89:D89"/>
     <mergeCell ref="B90:D90"/>
     <mergeCell ref="B91:D91"/>
     <mergeCell ref="B92:D92"/>
     <mergeCell ref="B93:D93"/>
-    <mergeCell ref="B94:D94"/>
     <mergeCell ref="B95:D95"/>
+    <mergeCell ref="B96:D96"/>
     <mergeCell ref="B97:D97"/>
     <mergeCell ref="B98:D98"/>
-    <mergeCell ref="B99:D99"/>
-    <mergeCell ref="B100:D100"/>
-    <mergeCell ref="B101:D102"/>
-    <mergeCell ref="E101:G101"/>
-    <mergeCell ref="I101:I102"/>
+    <mergeCell ref="B99:D100"/>
+    <mergeCell ref="E99:G99"/>
+    <mergeCell ref="I99:I100"/>
+    <mergeCell ref="B101:D101"/>
+    <mergeCell ref="B102:D102"/>
     <mergeCell ref="B103:D103"/>
-    <mergeCell ref="B104:D104"/>
-    <mergeCell ref="B105:D105"/>
-    <mergeCell ref="B112:D112"/>
-    <mergeCell ref="B113:D114"/>
-    <mergeCell ref="E113:G113"/>
-    <mergeCell ref="I113:I114"/>
+    <mergeCell ref="B110:D110"/>
+    <mergeCell ref="B111:D112"/>
+    <mergeCell ref="E111:G111"/>
+    <mergeCell ref="I111:I112"/>
+    <mergeCell ref="B113:D113"/>
+    <mergeCell ref="B114:D114"/>
     <mergeCell ref="B115:D115"/>
     <mergeCell ref="B116:D116"/>
-    <mergeCell ref="B117:D117"/>
     <mergeCell ref="B118:D118"/>
-    <mergeCell ref="B120:D120"/>
-    <mergeCell ref="B131:D131"/>
-    <mergeCell ref="B132:D133"/>
-    <mergeCell ref="E132:G132"/>
-    <mergeCell ref="I132:I133"/>
-    <mergeCell ref="B134:D134"/>
-    <mergeCell ref="B135:D135"/>
-    <mergeCell ref="B137:D137"/>
-    <mergeCell ref="B147:D147"/>
-    <mergeCell ref="B148:D148"/>
-    <mergeCell ref="B149:D149"/>
-    <mergeCell ref="B150:D150"/>
-    <mergeCell ref="B151:D151"/>
-    <mergeCell ref="B158:D158"/>
-    <mergeCell ref="B169:D169"/>
+    <mergeCell ref="B127:D128"/>
+    <mergeCell ref="E127:G127"/>
+    <mergeCell ref="I127:I128"/>
+    <mergeCell ref="B129:D129"/>
+    <mergeCell ref="B130:D130"/>
+    <mergeCell ref="B132:D132"/>
+    <mergeCell ref="B142:D142"/>
+    <mergeCell ref="B143:D143"/>
+    <mergeCell ref="B144:D144"/>
+    <mergeCell ref="B145:D145"/>
+    <mergeCell ref="B146:D146"/>
+    <mergeCell ref="B152:D152"/>
+    <mergeCell ref="B163:D163"/>
   </mergeCells>
   <printOptions headings="0" gridLines="0" horizontalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.64999999999999991" header="0.25" footer="0.25"/>
-  <pageSetup paperSize="9" scale="90" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="90" firstPageNumber="1" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="1" errors="displayed" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
     <oddHeader>&amp;R&amp;8&amp;D</oddHeader>
     <oddFooter>&amp;R&amp;8&amp;P</oddFooter>

</xml_diff>